<commit_message>
data: replace trade-area DB and add cafe video URL
</commit_message>
<xml_diff>
--- a/app/template_knowledge/sources/영상편집DB.xlsx
+++ b/app/template_knowledge/sources/영상편집DB.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R576131c6b8b6403e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R016037fba0e6416f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="Rfa4668d079244ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="Rcb4cf71566a44214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R23d6434092254068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="Rd5588dee259f4ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="R241bfb6c422a445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R706ad47ef9b14d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R85acde8afbde4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="R9faeec7798c44953"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R17c462851164430e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R95bbdf72f9994571"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R87395bafb1874d51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R8ab9419d8a5a4629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R0a17b4958cc84099"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R1428eea5ef8c4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R16f82cb6d0444ef1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R7e74f51c363a40be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="Ra76d2a1f66bb4f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="Rf10f84783210447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R17272ad391c340e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R5f2f7acb8f8441e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="R622f108746d049cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R2ceb10cae35f4c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R6100602d2eb54910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="Rab55d6eb79934e2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31958,8 +31958,12 @@
       <x:c r="F7" s="47" t="str">
         <x:v>카페 추천 리뷰 릴스</x:v>
       </x:c>
-      <x:c r="G7" s="47"/>
-      <x:c r="H7" s="47"/>
+      <x:c r="G7" s="47" t="str">
+        <x:v>https://www.youtube.com/shorts/OWnLiuJU8Ks</x:v>
+      </x:c>
+      <x:c r="H7" s="47" t="str">
+        <x:v>OWnLiuJU8Ks</x:v>
+      </x:c>
       <x:c r="I7" s="47" t="str">
         <x:v>PASS</x:v>
       </x:c>

</xml_diff>

<commit_message>
feat: add informational shortform shooting elements
</commit_message>
<xml_diff>
--- a/app/template_knowledge/sources/영상편집DB.xlsx
+++ b/app/template_knowledge/sources/영상편집DB.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R4651dc3642b1486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R6b681fbb4a2e4b47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R561d980d27e24494"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R8951591f35b14d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="Rfd4ead5a0ca247a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="Rf597362cdc9e4246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="Rc5b11f33bb374417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R113f0cb8c6cb483a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R30be0a5f15b6459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="Ra7a056af11d14ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R09ebc56dece64c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R7426b7047afc407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R0cc8b2d00f4c4926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R2032648c311c49f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R33393f5afa1243f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R2e1b16fa1d6845fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R5908d5be669743be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="Rba65ef4661e54f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R109d77a2b9e64612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="Rf0ea8f17fd0b49ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="Rd3df3d48fe764a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="Re9ef99df09b442b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="Rbfdc28e7f10b4a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="Rd5383b432b494061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R2f77975909b74c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R362a1cf81b04478d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03A_SHOOTING_ELEMENTS" sheetId="14" r:id="R0a5b31abfd4445a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -364,7 +365,7 @@
     <x:numFmt numFmtId="177" formatCode="0.0"/>
     <x:numFmt numFmtId="178" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -427,8 +428,19 @@
       <x:color theme="10"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -500,8 +512,38 @@
         <x:fgColor rgb="FFFFF3C9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="13">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -532,13 +574,103 @@
         <x:color rgb="FFCAD6DB"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="80">
+  <x:cellXfs count="115">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -775,6 +907,75 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="3">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -782,6 +983,24 @@
     <x:cellStyle name="하이퍼링크" xfId="2"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InformationalShootingElementsTable" displayName="InformationalShootingElementsTable" ref="A4:J8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="shooting_element_id"/>
+    <x:tableColumn id="2" name="guide_template_id"/>
+    <x:tableColumn id="3" name="challenge_id"/>
+    <x:tableColumn id="4" name="display_order"/>
+    <x:tableColumn id="5" name="title"/>
+    <x:tableColumn id="6" name="instruction"/>
+    <x:tableColumn id="7" name="minimum_recording_sec"/>
+    <x:tableColumn id="8" name="reference_segment_sequences"/>
+    <x:tableColumn id="9" name="validation_status"/>
+    <x:tableColumn id="10" name="template_status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35380,6 +35599,222 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="107" t="str">
+        <x:v>정보형 숏폼 촬영 요소</x:v>
+      </x:c>
+      <x:c r="B1" s="107"/>
+      <x:c r="C1" s="107"/>
+      <x:c r="D1" s="107"/>
+      <x:c r="E1" s="107"/>
+      <x:c r="F1" s="107"/>
+      <x:c r="G1" s="107"/>
+      <x:c r="H1" s="107"/>
+      <x:c r="I1" s="107"/>
+      <x:c r="J1" s="107"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="110" t="str">
+        <x:v>사용자에게는 최대 5개 요소만 제공하며, 내부 편집 컷은 shooting_element_id로 연결합니다.</x:v>
+      </x:c>
+      <x:c r="B2" s="110"/>
+      <x:c r="C2" s="110"/>
+      <x:c r="D2" s="110"/>
+      <x:c r="E2" s="110"/>
+      <x:c r="F2" s="110"/>
+      <x:c r="G2" s="110"/>
+      <x:c r="H2" s="110"/>
+      <x:c r="I2" s="110"/>
+      <x:c r="J2" s="110"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="112" t="str">
+        <x:v>shooting_element_id</x:v>
+      </x:c>
+      <x:c r="B4" s="113" t="str">
+        <x:v>guide_template_id</x:v>
+      </x:c>
+      <x:c r="C4" s="113" t="str">
+        <x:v>challenge_id</x:v>
+      </x:c>
+      <x:c r="D4" s="113" t="str">
+        <x:v>display_order</x:v>
+      </x:c>
+      <x:c r="E4" s="113" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="F4" s="113" t="str">
+        <x:v>instruction</x:v>
+      </x:c>
+      <x:c r="G4" s="113" t="str">
+        <x:v>minimum_recording_sec</x:v>
+      </x:c>
+      <x:c r="H4" s="113" t="str">
+        <x:v>reference_segment_sequences</x:v>
+      </x:c>
+      <x:c r="I4" s="113" t="str">
+        <x:v>validation_status</x:v>
+      </x:c>
+      <x:c r="J4" s="114" t="str">
+        <x:v>template_status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="98" t="str">
+        <x:v>ELEMENT_01</x:v>
+      </x:c>
+      <x:c r="B5" s="99" t="str">
+        <x:v>gt_cafe_recommendation_v2</x:v>
+      </x:c>
+      <x:c r="C5" s="99" t="str">
+        <x:v>cafe_recommendation_reels</x:v>
+      </x:c>
+      <x:c r="D5" s="99" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="99" t="str">
+        <x:v>제조 과정</x:v>
+      </x:c>
+      <x:c r="F5" s="99" t="str">
+        <x:v>준비와 추출 과정을 손동작이 보이게 길게 촬영하세요.</x:v>
+      </x:c>
+      <x:c r="G5" s="99" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H5" s="99" t="str">
+        <x:v>1,13,14,15,16,23</x:v>
+      </x:c>
+      <x:c r="I5" s="99" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J5" s="100" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="98" t="str">
+        <x:v>ELEMENT_02</x:v>
+      </x:c>
+      <x:c r="B6" s="99" t="str">
+        <x:v>gt_cafe_recommendation_v2</x:v>
+      </x:c>
+      <x:c r="C6" s="99" t="str">
+        <x:v>cafe_recommendation_reels</x:v>
+      </x:c>
+      <x:c r="D6" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E6" s="99" t="str">
+        <x:v>대표 메뉴</x:v>
+      </x:c>
+      <x:c r="F6" s="99" t="str">
+        <x:v>음료와 디저트 전체·세부 모습을 여러 각도로 촬영하세요.</x:v>
+      </x:c>
+      <x:c r="G6" s="99" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H6" s="99" t="str">
+        <x:v>2,3,9,10,11,12,17,20,21</x:v>
+      </x:c>
+      <x:c r="I6" s="99" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J6" s="100" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="98" t="str">
+        <x:v>ELEMENT_03</x:v>
+      </x:c>
+      <x:c r="B7" s="99" t="str">
+        <x:v>gt_cafe_recommendation_v2</x:v>
+      </x:c>
+      <x:c r="C7" s="99" t="str">
+        <x:v>cafe_recommendation_reels</x:v>
+      </x:c>
+      <x:c r="D7" s="99" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E7" s="99" t="str">
+        <x:v>체험과 전망</x:v>
+      </x:c>
+      <x:c r="F7" s="99" t="str">
+        <x:v>컵을 든 모습과 매장 밖 전망을 각각 길게 촬영하세요.</x:v>
+      </x:c>
+      <x:c r="G7" s="99" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H7" s="99" t="str">
+        <x:v>4,5,6,7,8</x:v>
+      </x:c>
+      <x:c r="I7" s="99" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J7" s="100" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="101" t="str">
+        <x:v>ELEMENT_04</x:v>
+      </x:c>
+      <x:c r="B8" s="102" t="str">
+        <x:v>gt_cafe_recommendation_v2</x:v>
+      </x:c>
+      <x:c r="C8" s="102" t="str">
+        <x:v>cafe_recommendation_reels</x:v>
+      </x:c>
+      <x:c r="D8" s="102" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="102" t="str">
+        <x:v>매장 분위기</x:v>
+      </x:c>
+      <x:c r="F8" s="102" t="str">
+        <x:v>창과 인테리어가 보이도록 매장 공간을 천천히 촬영하세요.</x:v>
+      </x:c>
+      <x:c r="G8" s="102" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H8" s="102" t="str">
+        <x:v>18,19,22</x:v>
+      </x:c>
+      <x:c r="I8" s="102" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J8" s="103" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radb0586adf194d94"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="14"/>
@@ -35614,6 +36049,7 @@
     <x:col min="7" max="7" width="30" customWidth="1"/>
     <x:col min="8" max="8" width="23.25" customWidth="1"/>
     <x:col min="9" max="9" width="24.1640625" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -35681,6 +36117,9 @@
       <x:c r="I4" s="1" t="str">
         <x:v>input_validation_status</x:v>
       </x:c>
+      <x:c r="J4" s="104" t="str">
+        <x:v>format_type</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -35710,6 +36149,9 @@
       <x:c r="I5" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
+      <x:c r="J5" s="63" t="str">
+        <x:v>밈</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -35739,6 +36181,9 @@
       <x:c r="I6" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
+      <x:c r="J6" s="63" t="str">
+        <x:v>챌린지</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -35765,6 +36210,9 @@
       <x:c r="H7" s="9"/>
       <x:c r="I7" s="9" t="str">
         <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J7" s="63" t="str">
+        <x:v>정보형</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -35778,9 +36226,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R2a5f6002b0d4479e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R705c2ea051e4455a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Raf6f7b73184e41e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R36632b385e214036"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R8af8ae4620e5467f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Ra0551073b25e4293"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -35813,6 +36261,7 @@
     <x:col min="23" max="23" width="28" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -35964,6 +36413,9 @@
       <x:c r="W4" s="64" t="str">
         <x:v>source_file_sha256</x:v>
       </x:c>
+      <x:c r="X4" s="105" t="str">
+        <x:v>shooting_element_id</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="78" customHeight="1">
       <x:c r="A5" s="65" t="str">
@@ -36035,6 +36487,7 @@
       <x:c r="W5" s="65" t="str">
         <x:v>61AAC25E38688E48000B399277828732BC201C1806FEFAA23419C76662B1B0E7</x:v>
       </x:c>
+      <x:c r="X5"/>
     </x:row>
     <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="65" t="str">
@@ -36106,6 +36559,7 @@
       <x:c r="W6" s="65" t="str">
         <x:v>61AAC25E38688E48000B399277828732BC201C1806FEFAA23419C76662B1B0E7</x:v>
       </x:c>
+      <x:c r="X6"/>
     </x:row>
     <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="65" t="str">
@@ -36177,6 +36631,7 @@
       <x:c r="W7" s="65" t="str">
         <x:v>61AAC25E38688E48000B399277828732BC201C1806FEFAA23419C76662B1B0E7</x:v>
       </x:c>
+      <x:c r="X7"/>
     </x:row>
     <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="65" t="str">
@@ -36242,6 +36697,7 @@
       <x:c r="W8" s="65" t="str">
         <x:v>61AAC25E38688E48000B399277828732BC201C1806FEFAA23419C76662B1B0E7</x:v>
       </x:c>
+      <x:c r="X8"/>
     </x:row>
     <x:row r="9" ht="78" customHeight="1">
       <x:c r="A9" s="65" t="str">
@@ -36313,6 +36769,7 @@
       <x:c r="W9" s="65" t="str">
         <x:v>B5BA6E95FE7BD0CD4F7A340EDC051E0BCCDF24D367ED1E60C495F1C96618A0B9</x:v>
       </x:c>
+      <x:c r="X9"/>
     </x:row>
     <x:row r="10" ht="78" customHeight="1">
       <x:c r="A10" s="65" t="str">
@@ -36380,6 +36837,7 @@
       <x:c r="W10" s="65" t="str">
         <x:v>B5BA6E95FE7BD0CD4F7A340EDC051E0BCCDF24D367ED1E60C495F1C96618A0B9</x:v>
       </x:c>
+      <x:c r="X10"/>
     </x:row>
     <x:row r="11" ht="78" customHeight="1">
       <x:c r="A11" s="65" t="str">
@@ -36447,6 +36905,7 @@
       <x:c r="W11" s="65" t="str">
         <x:v>B5BA6E95FE7BD0CD4F7A340EDC051E0BCCDF24D367ED1E60C495F1C96618A0B9</x:v>
       </x:c>
+      <x:c r="X11"/>
     </x:row>
     <x:row r="12" ht="78" customHeight="1">
       <x:c r="A12" s="65" t="str">
@@ -36514,6 +36973,7 @@
       <x:c r="W12" s="65" t="str">
         <x:v>B5BA6E95FE7BD0CD4F7A340EDC051E0BCCDF24D367ED1E60C495F1C96618A0B9</x:v>
       </x:c>
+      <x:c r="X12"/>
     </x:row>
     <x:row r="13" ht="78" customHeight="1">
       <x:c r="A13" s="65" t="str">
@@ -36585,6 +37045,7 @@
       <x:c r="W13" s="65" t="str">
         <x:v>B5BA6E95FE7BD0CD4F7A340EDC051E0BCCDF24D367ED1E60C495F1C96618A0B9</x:v>
       </x:c>
+      <x:c r="X13"/>
     </x:row>
     <x:row r="14" ht="78" customHeight="1">
       <x:c r="A14" s="65" t="str">
@@ -36656,6 +37117,9 @@
       <x:c r="W14" s="65" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
       </x:c>
+      <x:c r="X14" t="str">
+        <x:v>ELEMENT_01</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="78" customHeight="1">
       <x:c r="A15" s="65" t="str">
@@ -36727,6 +37191,9 @@
       <x:c r="W15" s="65" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
       </x:c>
+      <x:c r="X15" t="str">
+        <x:v>ELEMENT_02</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="78" customHeight="1">
       <x:c r="A16" s="65" t="str">
@@ -36798,6 +37265,9 @@
       <x:c r="W16" s="65" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
       </x:c>
+      <x:c r="X16" t="str">
+        <x:v>ELEMENT_01</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="78" customHeight="1">
       <x:c r="A17" s="65" t="str">
@@ -36869,6 +37339,9 @@
       <x:c r="W17" s="65" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
       </x:c>
+      <x:c r="X17" t="str">
+        <x:v>ELEMENT_03</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="78" customHeight="1">
       <x:c r="A18" s="65" t="str">
@@ -36940,6 +37413,9 @@
       <x:c r="W18" s="65" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
       </x:c>
+      <x:c r="X18" t="str">
+        <x:v>ELEMENT_04</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="78" customHeight="1">
       <x:c r="A19" s="69" t="str">
@@ -37010,6 +37486,9 @@
       </x:c>
       <x:c r="W19" s="69" t="str">
         <x:v>70A521B50E58B1355992AC47AEB7C36E7C98174A9826BEE007A464FD20ECA140</x:v>
+      </x:c>
+      <x:c r="X19" t="str">
+        <x:v>ELEMENT_04</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="78" customHeight="1">

</xml_diff>

<commit_message>
feat: refresh ranked video editing guides
</commit_message>
<xml_diff>
--- a/app/template_knowledge/sources/영상편집DB.xlsx
+++ b/app/template_knowledge/sources/영상편집DB.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R457d46e0091b4f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R1b75e9a3ea38480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R25d335b7020b41d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R04f7d9cc4e664e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R274557fdb13543bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R3ce23ae9300744ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="R696449c80e624539"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="Ra344ed7808d34229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="Raddf62cf79ea418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="R112e96942e894201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R316d4dee8fd741c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R96c9cb0ce0c44fb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R8b6fff9d59b247d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R2559efaf5987480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R723ce5923351474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="Rb7fe763e7bd64973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R9e0a4e0e15734cde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R5efd6aef886f4420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R0fcb1d9fe35340d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="R2300e1cb26c44df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R657d1f5689cb45d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R362a401d4c654592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="Ree13d59270e84394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="Rbd47d9c6a19349cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="Rf769d156e8204fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R4f30a5f5a4c54b63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -959,7 +959,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 두 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 5프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
+        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 세 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -1253,16 +1253,16 @@
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>실제 가이드 2종</x:v>
+        <x:v>실제 가이드 3종</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>주술회전 트랜지션 · 오츠카레 썸머 챌린지를 실제 레코드로 등록</x:v>
+        <x:v>주술회전 트랜지션 · 동그리오 챌린지 · 오츠카레 썸머 챌린지를 실제 레코드로 등록</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
         <x:v>02, 03, 12</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>12_SOURCE_GUIDES에 두 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
+        <x:v>12_SOURCE_GUIDES에 세 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26296,368 +26296,984 @@
       </x:c>
     </x:row>
     <x:row r="679" ht="18" customHeight="1">
-      <x:c r="A679"/>
-      <x:c r="B679"/>
-      <x:c r="C679"/>
-      <x:c r="D679"/>
-      <x:c r="E679"/>
-      <x:c r="F679"/>
-      <x:c r="G679"/>
-      <x:c r="H679"/>
-      <x:c r="I679"/>
-      <x:c r="J679"/>
-      <x:c r="K679"/>
+      <x:c r="A679" t="str">
+        <x:v>jujutsu20260830_line_0001</x:v>
+      </x:c>
+      <x:c r="B679" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C679" t="n">
+        <x:v>895</x:v>
+      </x:c>
+      <x:c r="D679" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E679" t="str">
+        <x:v>SUMMARY</x:v>
+      </x:c>
+      <x:c r="F679" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G679" t="str">
+        <x:v>- source_url: https://www.youtube.com/shorts/Aa-CGr9-c8E; 14초, 8컷, 4개 SETUP/REVEAL 매치컷 쌍, confidence=0.98, 촬영 난이도 ★★.</x:v>
+      </x:c>
+      <x:c r="H679" t="str">
+        <x:v>주술회전_1프레임분석.json</x:v>
+      </x:c>
+      <x:c r="I679" t="str">
+        <x:v>6868F640E082BDCFE1616CAF43F36267706D571358838896B5CDC74CC6646F31</x:v>
+      </x:c>
+      <x:c r="J679" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K679" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="680" ht="18" customHeight="1">
-      <x:c r="A680"/>
-      <x:c r="B680"/>
-      <x:c r="C680"/>
-      <x:c r="D680"/>
-      <x:c r="E680"/>
-      <x:c r="F680"/>
-      <x:c r="G680"/>
-      <x:c r="H680"/>
-      <x:c r="I680"/>
-      <x:c r="J680"/>
-      <x:c r="K680"/>
+      <x:c r="A680" t="str">
+        <x:v>jujutsu20260830_line_0002</x:v>
+      </x:c>
+      <x:c r="B680" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C680" t="n">
+        <x:v>896</x:v>
+      </x:c>
+      <x:c r="D680" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E680" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F680" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G680" t="str">
+        <x:v>- S01 0-1500ms HOOK_SETUP: 인물 A가 고정 미디엄 구도에서 빈손 시그니처 포즈에 진입해 안정적으로 유지</x:v>
+      </x:c>
+      <x:c r="H680" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I680" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J680" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K680" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="681" ht="18" customHeight="1">
-      <x:c r="A681"/>
-      <x:c r="B681"/>
-      <x:c r="C681"/>
-      <x:c r="D681"/>
-      <x:c r="E681"/>
-      <x:c r="F681"/>
-      <x:c r="G681"/>
-      <x:c r="H681"/>
-      <x:c r="I681"/>
-      <x:c r="J681"/>
-      <x:c r="K681"/>
+      <x:c r="A681" t="str">
+        <x:v>jujutsu20260830_line_0003</x:v>
+      </x:c>
+      <x:c r="B681" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C681" t="n">
+        <x:v>897</x:v>
+      </x:c>
+      <x:c r="D681" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E681" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F681" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G681" t="str">
+        <x:v>- S02 1500-3500ms MAGIC_REVEAL: S01과 동일 포즈·구도에서 인물 A의 손에 실제 음료가 나타난 상태로 시작해 결과를 유지</x:v>
+      </x:c>
+      <x:c r="H681" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I681" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J681" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K681" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="682" ht="18" customHeight="1">
-      <x:c r="A682"/>
-      <x:c r="B682"/>
-      <x:c r="C682"/>
-      <x:c r="D682"/>
-      <x:c r="E682"/>
-      <x:c r="F682"/>
-      <x:c r="G682"/>
-      <x:c r="H682"/>
-      <x:c r="I682"/>
-      <x:c r="J682"/>
-      <x:c r="K682"/>
+      <x:c r="A682" t="str">
+        <x:v>jujutsu20260830_line_0004</x:v>
+      </x:c>
+      <x:c r="B682" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C682" t="n">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="D682" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E682" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F682" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G682" t="str">
+        <x:v>- S03 3500-5000ms SETUP: 인물 B가 같은 고정 카메라에서 새로운 빈손 포즈를 취하고 안정 구간을 유지</x:v>
+      </x:c>
+      <x:c r="H682" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I682" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J682" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K682" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="683" ht="18" customHeight="1">
-      <x:c r="A683"/>
-      <x:c r="B683"/>
-      <x:c r="C683"/>
-      <x:c r="D683"/>
-      <x:c r="E683"/>
-      <x:c r="F683"/>
-      <x:c r="G683"/>
-      <x:c r="H683"/>
-      <x:c r="I683"/>
-      <x:c r="J683"/>
-      <x:c r="K683"/>
+      <x:c r="A683" t="str">
+        <x:v>jujutsu20260830_line_0005</x:v>
+      </x:c>
+      <x:c r="B683" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C683" t="n">
+        <x:v>899</x:v>
+      </x:c>
+      <x:c r="D683" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E683" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F683" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G683" t="str">
+        <x:v>- S04 5000-7000ms MAGIC_REVEAL: S03과 동일 포즈·구도에서 인물 B의 손에 다른 음료가 나타난 상태로 전환</x:v>
+      </x:c>
+      <x:c r="H683" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I683" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J683" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K683" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="684" ht="18" customHeight="1">
-      <x:c r="A684"/>
-      <x:c r="B684"/>
-      <x:c r="C684"/>
-      <x:c r="D684"/>
-      <x:c r="E684"/>
-      <x:c r="F684"/>
-      <x:c r="G684"/>
-      <x:c r="H684"/>
-      <x:c r="I684"/>
-      <x:c r="J684"/>
-      <x:c r="K684"/>
+      <x:c r="A684" t="str">
+        <x:v>jujutsu20260830_line_0006</x:v>
+      </x:c>
+      <x:c r="B684" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C684" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="D684" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E684" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F684" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G684" t="str">
+        <x:v>- S05 7000-8500ms SETUP: 인물 A가 다시 등장해 케이크 공개 전 새 빈손 포즈를 안정적으로 유지</x:v>
+      </x:c>
+      <x:c r="H684" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I684" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J684" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K684" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="685" ht="18" customHeight="1">
-      <x:c r="A685"/>
-      <x:c r="B685"/>
-      <x:c r="C685"/>
-      <x:c r="D685"/>
-      <x:c r="E685"/>
-      <x:c r="F685"/>
-      <x:c r="G685"/>
-      <x:c r="H685"/>
-      <x:c r="I685"/>
-      <x:c r="J685"/>
-      <x:c r="K685"/>
+      <x:c r="A685" t="str">
+        <x:v>jujutsu20260830_line_0007</x:v>
+      </x:c>
+      <x:c r="B685" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C685" t="n">
+        <x:v>901</x:v>
+      </x:c>
+      <x:c r="D685" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E685" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F685" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G685" t="str">
+        <x:v>- S06 8500-10500ms MAGIC_REVEAL: S05와 동일 포즈·구도에서 인물 A가 실제 케이크 접시를 든 상태로 시작</x:v>
+      </x:c>
+      <x:c r="H685" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I685" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J685" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K685" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="686" ht="18" customHeight="1">
-      <x:c r="A686"/>
-      <x:c r="B686"/>
-      <x:c r="C686"/>
-      <x:c r="D686"/>
-      <x:c r="E686"/>
-      <x:c r="F686"/>
-      <x:c r="G686"/>
-      <x:c r="H686"/>
-      <x:c r="I686"/>
-      <x:c r="J686"/>
-      <x:c r="K686"/>
+      <x:c r="A686" t="str">
+        <x:v>jujutsu20260830_line_0008</x:v>
+      </x:c>
+      <x:c r="B686" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C686" t="n">
+        <x:v>902</x:v>
+      </x:c>
+      <x:c r="D686" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E686" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F686" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G686" t="str">
+        <x:v>- S07 10500-12000ms SETUP: 인물 B가 마지막 공개를 위한 빈손 포즈를 취하고 배경·카메라를 고정</x:v>
+      </x:c>
+      <x:c r="H686" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I686" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J686" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K686" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="687" ht="18" customHeight="1">
-      <x:c r="A687"/>
-      <x:c r="B687"/>
-      <x:c r="C687"/>
-      <x:c r="D687"/>
-      <x:c r="E687"/>
-      <x:c r="F687"/>
-      <x:c r="G687"/>
-      <x:c r="H687"/>
-      <x:c r="I687"/>
-      <x:c r="J687"/>
-      <x:c r="K687"/>
+      <x:c r="A687" t="str">
+        <x:v>jujutsu20260830_line_0009</x:v>
+      </x:c>
+      <x:c r="B687" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C687" t="n">
+        <x:v>903</x:v>
+      </x:c>
+      <x:c r="D687" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E687" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F687" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G687" t="str">
+        <x:v>- S08 12000-14000ms MAGIC_REVEAL: S07과 동일 포즈·구도에서 실제 빵 접시가 나타난 상태로 전환해 아웃트로 유지</x:v>
+      </x:c>
+      <x:c r="H687" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I687" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J687" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K687" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="688" ht="18" customHeight="1">
-      <x:c r="A688"/>
-      <x:c r="B688"/>
-      <x:c r="C688"/>
-      <x:c r="D688"/>
-      <x:c r="E688"/>
-      <x:c r="F688"/>
-      <x:c r="G688"/>
-      <x:c r="H688"/>
-      <x:c r="I688"/>
-      <x:c r="J688"/>
-      <x:c r="K688"/>
+      <x:c r="A688" t="str">
+        <x:v>jujutsu20260830_line_0010</x:v>
+      </x:c>
+      <x:c r="B688" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C688" t="n">
+        <x:v>904</x:v>
+      </x:c>
+      <x:c r="D688" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E688" t="str">
+        <x:v>AUDIO_SYNC</x:v>
+      </x:c>
+      <x:c r="F688" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G688" t="str">
+        <x:v>- reveal_sfx_markers_ms: 1500, 5000, 8500, 12000; 모든 MAGIC_REVEAL 첫 프레임을 타격점에 정렬.</x:v>
+      </x:c>
+      <x:c r="H688" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I688" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J688" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K688" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="689" ht="18" customHeight="1">
-      <x:c r="A689"/>
-      <x:c r="B689"/>
-      <x:c r="C689"/>
-      <x:c r="D689"/>
-      <x:c r="E689"/>
-      <x:c r="F689"/>
-      <x:c r="G689"/>
-      <x:c r="H689"/>
-      <x:c r="I689"/>
-      <x:c r="J689"/>
-      <x:c r="K689"/>
+      <x:c r="A689" t="str">
+        <x:v>jujutsu20260830_line_0011</x:v>
+      </x:c>
+      <x:c r="B689" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C689" t="n">
+        <x:v>905</x:v>
+      </x:c>
+      <x:c r="D689" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E689" t="str">
+        <x:v>MATCH_RULE</x:v>
+      </x:c>
+      <x:c r="F689" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G689" t="str">
+        <x:v>- 각 SETUP/REVEAL 쌍은 동일 인물·카메라·배경·포즈를 유지하고 SETUP에는 아이템이 없어야 하며 REVEAL에는 명확히 보여야 함.</x:v>
+      </x:c>
+      <x:c r="H689" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I689" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J689" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K689" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="690" ht="18" customHeight="1">
-      <x:c r="A690"/>
-      <x:c r="B690"/>
-      <x:c r="C690"/>
-      <x:c r="D690"/>
-      <x:c r="E690"/>
-      <x:c r="F690"/>
-      <x:c r="G690"/>
-      <x:c r="H690"/>
-      <x:c r="I690"/>
-      <x:c r="J690"/>
-      <x:c r="K690"/>
+      <x:c r="A690" t="str">
+        <x:v>jujutsu20260830_line_0012</x:v>
+      </x:c>
+      <x:c r="B690" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C690" t="n">
+        <x:v>906</x:v>
+      </x:c>
+      <x:c r="D690" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E690" t="str">
+        <x:v>OVERLAY</x:v>
+      </x:c>
+      <x:c r="F690" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G690" t="str">
+        <x:v>- 별도 자막·애니메이션 오버레이 없음. 플랫폼 UI와 레퍼런스 오디오는 편집 요소로 복제하지 않음.</x:v>
+      </x:c>
+      <x:c r="H690" t="str">
+        <x:v>주술회전_1프레임분석.json</x:v>
+      </x:c>
+      <x:c r="I690" t="str">
+        <x:v>6868F640E082BDCFE1616CAF43F36267706D571358838896B5CDC74CC6646F31</x:v>
+      </x:c>
+      <x:c r="J690" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K690" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="691" ht="18" customHeight="1">
-      <x:c r="A691"/>
-      <x:c r="B691"/>
-      <x:c r="C691"/>
-      <x:c r="D691"/>
-      <x:c r="E691"/>
-      <x:c r="F691"/>
-      <x:c r="G691"/>
-      <x:c r="H691"/>
-      <x:c r="I691"/>
-      <x:c r="J691"/>
-      <x:c r="K691"/>
+      <x:c r="A691" t="str">
+        <x:v>jujutsu20260830_line_0013</x:v>
+      </x:c>
+      <x:c r="B691" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C691" t="n">
+        <x:v>907</x:v>
+      </x:c>
+      <x:c r="D691" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E691" t="str">
+        <x:v>VALIDATION</x:v>
+      </x:c>
+      <x:c r="F691" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G691" t="str">
+        <x:v>- hard_fail: 카메라 이동, 배경/인물 불일치, SETUP 아이템 노출, REVEAL 아이템 미노출, SFX 비동기, 경계 디졸브/페이드.</x:v>
+      </x:c>
+      <x:c r="H691" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I691" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J691" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K691" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="692" ht="18" customHeight="1">
-      <x:c r="A692"/>
-      <x:c r="B692"/>
-      <x:c r="C692"/>
-      <x:c r="D692"/>
-      <x:c r="E692"/>
-      <x:c r="F692"/>
-      <x:c r="G692"/>
-      <x:c r="H692"/>
-      <x:c r="I692"/>
-      <x:c r="J692"/>
-      <x:c r="K692"/>
+      <x:c r="A692" t="str">
+        <x:v>jujutsu20260830_line_0014</x:v>
+      </x:c>
+      <x:c r="B692" t="str">
+        <x:v>uploaded_jujutsu_json_20260830</x:v>
+      </x:c>
+      <x:c r="C692" t="n">
+        <x:v>908</x:v>
+      </x:c>
+      <x:c r="D692" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="E692" t="str">
+        <x:v>PROVENANCE</x:v>
+      </x:c>
+      <x:c r="F692" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G692" t="str">
+        <x:v>- 포즈/배경 정렬 점수·안정 구간 탐색·대체 테이크·미세 crop/translation 복구를 추가하되 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="H692" t="str">
+        <x:v>주술회전_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I692" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
+      <x:c r="J692" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="K692" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="693" ht="18" customHeight="1">
-      <x:c r="A693"/>
-      <x:c r="B693"/>
-      <x:c r="C693"/>
-      <x:c r="D693"/>
-      <x:c r="E693"/>
-      <x:c r="F693"/>
-      <x:c r="G693"/>
-      <x:c r="H693"/>
-      <x:c r="I693"/>
-      <x:c r="J693"/>
-      <x:c r="K693"/>
+      <x:c r="A693" t="str">
+        <x:v>donggeurio20260830_line_0001</x:v>
+      </x:c>
+      <x:c r="B693" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C693" t="n">
+        <x:v>909</x:v>
+      </x:c>
+      <x:c r="D693" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E693" t="str">
+        <x:v>SUMMARY</x:v>
+      </x:c>
+      <x:c r="F693" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G693" t="str">
+        <x:v>- source_url: https://www.youtube.com/shorts/iWyRoIJheV4; 실측 12.067초, 7컷 웜톤 카페 브이로그, shooting_difficulty: ★★, confidence=0.95.</x:v>
+      </x:c>
+      <x:c r="H693" t="str">
+        <x:v>동그리오_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I693" t="str">
+        <x:v>F8C3D8926CE141C84DF9C8077E82B5ABB6A90162A4E8BAF689277EDA85400A71</x:v>
+      </x:c>
+      <x:c r="J693" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K693" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="694" ht="18" customHeight="1">
-      <x:c r="A694"/>
-      <x:c r="B694"/>
-      <x:c r="C694"/>
-      <x:c r="D694"/>
-      <x:c r="E694"/>
-      <x:c r="F694"/>
-      <x:c r="G694"/>
-      <x:c r="H694"/>
-      <x:c r="I694"/>
-      <x:c r="J694"/>
-      <x:c r="K694"/>
+      <x:c r="A694" t="str">
+        <x:v>donggeurio20260830_line_0002</x:v>
+      </x:c>
+      <x:c r="B694" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C694" t="n">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="D694" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E694" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F694" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G694" t="str">
+        <x:v>- S01 0-1033ms HOOK: 안정적인 벽면·공간 디테일을 고정 구도로 보여주고 중앙 프로젝트 타이틀 배치</x:v>
+      </x:c>
+      <x:c r="H694" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I694" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J694" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K694" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="695" ht="18" customHeight="1">
-      <x:c r="A695"/>
-      <x:c r="B695"/>
-      <x:c r="C695"/>
-      <x:c r="D695"/>
-      <x:c r="E695"/>
-      <x:c r="F695"/>
-      <x:c r="G695"/>
-      <x:c r="H695"/>
-      <x:c r="I695"/>
-      <x:c r="J695"/>
-      <x:c r="K695"/>
+      <x:c r="A695" t="str">
+        <x:v>donggeurio20260830_line_0003</x:v>
+      </x:c>
+      <x:c r="B695" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C695" t="n">
+        <x:v>911</x:v>
+      </x:c>
+      <x:c r="D695" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E695" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F695" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G695" t="str">
+        <x:v>- S02 1033-3767ms REVEAL: 메뉴 전체가 보이는 탑다운/하이앵글 샷에 1.00→1.05 선형 줌인과 하단 보조 텍스트 적용</x:v>
+      </x:c>
+      <x:c r="H695" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I695" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J695" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K695" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="696" ht="18" customHeight="1">
-      <x:c r="A696"/>
-      <x:c r="B696"/>
-      <x:c r="C696"/>
-      <x:c r="D696"/>
-      <x:c r="E696"/>
-      <x:c r="F696"/>
-      <x:c r="G696"/>
-      <x:c r="H696"/>
-      <x:c r="I696"/>
-      <x:c r="J696"/>
-      <x:c r="K696"/>
+      <x:c r="A696" t="str">
+        <x:v>donggeurio20260830_line_0004</x:v>
+      </x:c>
+      <x:c r="B696" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C696" t="n">
+        <x:v>912</x:v>
+      </x:c>
+      <x:c r="D696" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E696" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F696" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G696" t="str">
+        <x:v>- S03 3767-4700ms AMBIENCE: 조명·좌석·인테리어를 보여주는 가장 매끄러운 우향 팬/측면 이동 구간 선택</x:v>
+      </x:c>
+      <x:c r="H696" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I696" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J696" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K696" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="697" ht="18" customHeight="1">
-      <x:c r="A697"/>
-      <x:c r="B697"/>
-      <x:c r="C697"/>
-      <x:c r="D697"/>
-      <x:c r="E697"/>
-      <x:c r="F697"/>
-      <x:c r="G697"/>
-      <x:c r="H697"/>
-      <x:c r="I697"/>
-      <x:c r="J697"/>
-      <x:c r="K697"/>
+      <x:c r="A697" t="str">
+        <x:v>donggeurio20260830_line_0005</x:v>
+      </x:c>
+      <x:c r="B697" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C697" t="n">
+        <x:v>913</x:v>
+      </x:c>
+      <x:c r="D697" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E697" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F697" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G697" t="str">
+        <x:v>- S04 4700-7000ms ACTION: 손이나 도구가 음식에 개입하는 클로즈업에서 동작 시작·피크·종료를 보존</x:v>
+      </x:c>
+      <x:c r="H697" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I697" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J697" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K697" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="698" ht="18" customHeight="1">
-      <x:c r="A698"/>
-      <x:c r="B698"/>
-      <x:c r="C698"/>
-      <x:c r="D698"/>
-      <x:c r="E698"/>
-      <x:c r="F698"/>
-      <x:c r="G698"/>
-      <x:c r="H698"/>
-      <x:c r="I698"/>
-      <x:c r="J698"/>
-      <x:c r="K698"/>
+      <x:c r="A698" t="str">
+        <x:v>donggeurio20260830_line_0006</x:v>
+      </x:c>
+      <x:c r="B698" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C698" t="n">
+        <x:v>914</x:v>
+      </x:c>
+      <x:c r="D698" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E698" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F698" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G698" t="str">
+        <x:v>- S05 7000-8333ms ACTION_HIGHLIGHT: 포크/나이프로 음식을 자르거나 분리하는 핵심 순간을 타이트한 클로즈업으로 강조</x:v>
+      </x:c>
+      <x:c r="H698" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I698" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J698" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K698" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="699" ht="18" customHeight="1">
-      <x:c r="A699"/>
-      <x:c r="B699"/>
-      <x:c r="C699"/>
-      <x:c r="D699"/>
-      <x:c r="E699"/>
-      <x:c r="F699"/>
-      <x:c r="G699"/>
-      <x:c r="H699"/>
-      <x:c r="I699"/>
-      <x:c r="J699"/>
-      <x:c r="K699"/>
+      <x:c r="A699" t="str">
+        <x:v>donggeurio20260830_line_0007</x:v>
+      </x:c>
+      <x:c r="B699" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C699" t="n">
+        <x:v>915</x:v>
+      </x:c>
+      <x:c r="D699" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E699" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F699" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G699" t="str">
+        <x:v>- S06 8333-9633ms LOCATION: 매장 외관·간판·입구 등 장소를 식별할 수 있는 구도를 짧게 제시하고 지원될 때만 미세 줌</x:v>
+      </x:c>
+      <x:c r="H699" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I699" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J699" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K699" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="700" ht="18" customHeight="1">
-      <x:c r="A700"/>
-      <x:c r="B700"/>
-      <x:c r="C700"/>
-      <x:c r="D700"/>
-      <x:c r="E700"/>
-      <x:c r="F700"/>
-      <x:c r="G700"/>
-      <x:c r="H700"/>
-      <x:c r="I700"/>
-      <x:c r="J700"/>
-      <x:c r="K700"/>
+      <x:c r="A700" t="str">
+        <x:v>donggeurio20260830_line_0008</x:v>
+      </x:c>
+      <x:c r="B700" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C700" t="n">
+        <x:v>916</x:v>
+      </x:c>
+      <x:c r="D700" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E700" t="str">
+        <x:v>SHOT</x:v>
+      </x:c>
+      <x:c r="F700" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G700" t="str">
+        <x:v>- S07 9633-12067ms OUTRO: 비비기·들어올리기·떠먹기 등 최종 음식 클로즈업에 1.05→1.00 ease-out 줌아웃</x:v>
+      </x:c>
+      <x:c r="H700" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I700" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J700" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K700" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="701" ht="18" customHeight="1">
-      <x:c r="A701"/>
-      <x:c r="B701"/>
-      <x:c r="C701"/>
-      <x:c r="D701"/>
-      <x:c r="E701"/>
-      <x:c r="F701"/>
-      <x:c r="G701"/>
-      <x:c r="H701"/>
-      <x:c r="I701"/>
-      <x:c r="J701"/>
-      <x:c r="K701"/>
+      <x:c r="A701" t="str">
+        <x:v>donggeurio20260830_line_0009</x:v>
+      </x:c>
+      <x:c r="B701" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C701" t="n">
+        <x:v>917</x:v>
+      </x:c>
+      <x:c r="D701" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E701" t="str">
+        <x:v>TIMELINE</x:v>
+      </x:c>
+      <x:c r="F701" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G701" t="str">
+        <x:v>- measured_boundaries_ms: 0,1033,3767,4700,7000,8333,9633,12067. 실행 시간축은 MP4 실측 경계를, 의미 라벨은 분석 JSON을 우선.</x:v>
+      </x:c>
+      <x:c r="H701" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I701" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J701" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K701" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="702" ht="18" customHeight="1">
-      <x:c r="A702"/>
-      <x:c r="B702"/>
-      <x:c r="C702"/>
-      <x:c r="D702"/>
-      <x:c r="E702"/>
-      <x:c r="F702"/>
-      <x:c r="G702"/>
-      <x:c r="H702"/>
-      <x:c r="I702"/>
-      <x:c r="J702"/>
-      <x:c r="K702"/>
+      <x:c r="A702" t="str">
+        <x:v>donggeurio20260830_line_0010</x:v>
+      </x:c>
+      <x:c r="B702" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C702" t="n">
+        <x:v>918</x:v>
+      </x:c>
+      <x:c r="D702" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E702" t="str">
+        <x:v>COLOR</x:v>
+      </x:c>
+      <x:c r="F702" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G702" t="str">
+        <x:v>- WARM tone; contrast/saturation +10~15%. 정확한 temperature 값은 COLOR.WARM_VLOG.TEMPERATURE 정책에서 해결.</x:v>
+      </x:c>
+      <x:c r="H702" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I702" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J702" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K702" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="703" ht="18" customHeight="1">
-      <x:c r="A703"/>
-      <x:c r="B703"/>
-      <x:c r="C703"/>
-      <x:c r="D703"/>
-      <x:c r="E703"/>
-      <x:c r="F703"/>
-      <x:c r="G703"/>
-      <x:c r="H703"/>
-      <x:c r="I703"/>
-      <x:c r="J703"/>
-      <x:c r="K703"/>
+      <x:c r="A703" t="str">
+        <x:v>donggeurio20260830_line_0011</x:v>
+      </x:c>
+      <x:c r="B703" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C703" t="n">
+        <x:v>919</x:v>
+      </x:c>
+      <x:c r="D703" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E703" t="str">
+        <x:v>OVERLAY</x:v>
+      </x:c>
+      <x:c r="F703" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G703" t="str">
+        <x:v>- S01 중앙 타이틀, S02 하단 보조 텍스트. 레퍼런스 상호·핸들은 복제하지 않고 사용자 프로젝트 메타데이터로 교체.</x:v>
+      </x:c>
+      <x:c r="H703" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I703" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J703" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K703" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="704" ht="18" customHeight="1">
-      <x:c r="A704"/>
-      <x:c r="B704"/>
-      <x:c r="C704"/>
-      <x:c r="D704"/>
-      <x:c r="E704"/>
-      <x:c r="F704"/>
-      <x:c r="G704"/>
-      <x:c r="H704"/>
-      <x:c r="I704"/>
-      <x:c r="J704"/>
-      <x:c r="K704"/>
+      <x:c r="A704" t="str">
+        <x:v>donggeurio20260830_line_0012</x:v>
+      </x:c>
+      <x:c r="B704" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C704" t="n">
+        <x:v>920</x:v>
+      </x:c>
+      <x:c r="D704" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E704" t="str">
+        <x:v>AUDIO_SYNC</x:v>
+      </x:c>
+      <x:c r="F704" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G704" t="str">
+        <x:v>- BEAT_SYNC_MUSIC; 의미 앵커를 훼손하지 않는 범위에서 인접 강한 onset에 컷을 스냅. 플랫폼 음원은 사용자가 추가.</x:v>
+      </x:c>
+      <x:c r="H704" t="str">
+        <x:v>동그리오_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I704" t="str">
+        <x:v>F8C3D8926CE141C84DF9C8077E82B5ABB6A90162A4E8BAF689277EDA85400A71</x:v>
+      </x:c>
+      <x:c r="J704" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K704" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="705" ht="18" customHeight="1">
-      <x:c r="A705"/>
-      <x:c r="B705"/>
-      <x:c r="C705"/>
-      <x:c r="D705"/>
-      <x:c r="E705"/>
-      <x:c r="F705"/>
-      <x:c r="G705"/>
-      <x:c r="H705"/>
-      <x:c r="I705"/>
-      <x:c r="J705"/>
-      <x:c r="K705"/>
+      <x:c r="A705" t="str">
+        <x:v>donggeurio20260830_line_0013</x:v>
+      </x:c>
+      <x:c r="B705" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C705" t="n">
+        <x:v>921</x:v>
+      </x:c>
+      <x:c r="D705" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E705" t="str">
+        <x:v>PARAMETER_POLICY</x:v>
+      </x:c>
+      <x:c r="F705" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G705" t="str">
+        <x:v>- 미해결 키: COLOR.WARM_VLOG.TEMPERATURE, CAMERA.SLIGHT_ZOOM.DEFAULT, TRANSITION.FADE_OUT.DEFAULT_DURATION_MS.</x:v>
+      </x:c>
+      <x:c r="H705" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I705" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J705" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K705" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="706" ht="18" customHeight="1">
-      <x:c r="A706"/>
-      <x:c r="B706"/>
-      <x:c r="C706"/>
-      <x:c r="D706"/>
-      <x:c r="E706"/>
-      <x:c r="F706"/>
-      <x:c r="G706"/>
-      <x:c r="H706"/>
-      <x:c r="I706"/>
-      <x:c r="J706"/>
-      <x:c r="K706"/>
+      <x:c r="A706" t="str">
+        <x:v>donggeurio20260830_line_0014</x:v>
+      </x:c>
+      <x:c r="B706" t="str">
+        <x:v>uploaded_donggeurio_json_20260830</x:v>
+      </x:c>
+      <x:c r="C706" t="n">
+        <x:v>922</x:v>
+      </x:c>
+      <x:c r="D706" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="E706" t="str">
+        <x:v>VALIDATION</x:v>
+      </x:c>
+      <x:c r="F706" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G706" t="str">
+        <x:v>- 7개 슬롯, 컷 경계 단조 증가, 전체 12067±34ms, 액션 앵커 보존, 속도 범위 준수, 레퍼런스 브랜드 미복제.</x:v>
+      </x:c>
+      <x:c r="H706" t="str">
+        <x:v>동그리오_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I706" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
+      <x:c r="J706" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K706" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="707" ht="18" customHeight="1">
       <x:c r="A707"/>
@@ -32629,7 +33245,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 두 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 2위는 공란으로 유지하며 다른 순위를 당겨 채우지 않습니다.</x:v>
+        <x:v>승인된 세 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 1·2·3위를 유지하며 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -32660,10 +33276,10 @@
         <x:v>챌린지 입력</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>랭킹 1위와 3위만 유지하며 2위는 공란</x:v>
+        <x:v>주술회전 1위·동그리오 2위·오츠카레 썸머 3위</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>02_INPUT_GUIDES</x:v>
@@ -32674,10 +33290,10 @@
         <x:v>전체 가이드 템플릿 구간</x:v>
       </x:c>
       <x:c r="B6" s="5" t="n">
-        <x:v>54</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>삭제 대상 제거 후 남은 03_GUIDE_TEMPLATES 데이터 행</x:v>
+        <x:v>버전 이력을 포함한 03_GUIDE_TEMPLATES 데이터 행</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -32769,13 +33385,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>5프레임 분석 근거</x:v>
+        <x:v>프레임 분석 실행 구간</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>152</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>주술회전 75 + 오츠카레 썸머 77블록을 03 실행 구간에 흡수</x:v>
+        <x:v>기존 152개 블록 + 주술회전 8컷 + 동그리오 7컷의 신규 JSON 근거</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -32783,13 +33399,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>주술회전 v4 실행 구간</x:v>
+        <x:v>주술회전 v5 실행 구간</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>F0-F371을 비중첩 세팅/블러/리빌/홀드/루프 단위로 분해한 실행 템플릿</x:v>
+        <x:v>0~14초 SETUP/REVEAL 4쌍의 ACTIVE 8컷 템플릿</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -32811,13 +33427,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>카페 추천 리뷰 v2 실행 구간</x:v>
+        <x:v>동그리오 v1 실행 구간</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:v>23</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>F0-F304를 컷·자막 상태·무자막 gap·엔드카드·루프 프리픽스 기준 23개 비중첩 구간으로 분해</x:v>
+        <x:v>실측 0~12.067초의 훅·메뉴·공간·액션·외관·아웃트로 7컷</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -32863,7 +33479,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 주술회전·오츠카레 썸머 가이드의 실제 업로드 MP4 정밀 분석을 유지합니다. rank 1과 3을 보존하고 rank 2는 공란으로 둡니다.</x:v>
+        <x:v>승인된 주술회전·동그리오·오츠카레 썸머 가이드를 유지합니다. rank 1·2·3을 보존하고 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -32926,10 +33542,10 @@
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>uploaded_guide_videos_20260824</x:v>
-      </x:c>
-      <x:c r="B5" s="118" t="str">
-        <x:v>2026-08-24T22:00:00</x:v>
+        <x:v>uploaded_analysis_json_20260830</x:v>
+      </x:c>
+      <x:c r="B5" s="118" t="n">
+        <x:v>46264.395833333336</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
         <x:v>jujutsu_transition</x:v>
@@ -32947,7 +33563,7 @@
         <x:v>https://www.youtube.com/shorts/Aa-CGr9-c8E</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Yc7ZjC0n7oY</x:v>
+        <x:v>Aa-CGr9-c8E</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
         <x:v>PASS</x:v>
@@ -32961,50 +33577,73 @@
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>uploaded_guide_videos_20260824</x:v>
-      </x:c>
-      <x:c r="B6" s="118" t="str">
-        <x:v>2026-08-24T22:00:00</x:v>
+        <x:v>uploaded_analysis_json_20260830</x:v>
+      </x:c>
+      <x:c r="B6" s="118" t="n">
+        <x:v>46264.395833333336</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>otsukare_summer_challenge</x:v>
+        <x:v>donggeurio_challenge</x:v>
       </x:c>
       <x:c r="D6" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>오츠카레 썸머 챌린지</x:v>
+        <x:v>동그리오 챌린지</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>오츠카레 썸머 챌린지</x:v>
+        <x:v>동그리오 챌린지</x:v>
       </x:c>
       <x:c r="G6" s="30" t="str">
-        <x:v>https://www.youtube.com/shorts/e-dU9yQfmik?si=fGCn4wuBsTEm2Q-p</x:v>
+        <x:v>https://www.youtube.com/shorts/iWyRoIJheV4</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>e-dU9yQfmik</x:v>
+        <x:v>iWyRoIJheV4</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="J6" s="63" t="str">
+        <x:v>food</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>정보형</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
+      <x:c r="A7" t="str">
+        <x:v>uploaded_guide_videos_20260824</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>2026-08-24T22:00:00</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>otsukare_summer_challenge</x:v>
+      </x:c>
+      <x:c r="D7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>오츠카레 썸머 챌린지</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>오츠카레 썸머 챌린지</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>https://www.youtube.com/shorts/e-dU9yQfmik?si=fGCn4wuBsTEm2Q-p</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>e-dU9yQfmik</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
         <x:v>challenge</x:v>
       </x:c>
-      <x:c r="K6" t="str">
+      <x:c r="K7" t="str">
         <x:v>챌린지</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="38" customHeight="1">
-      <x:c r="A7"/>
-      <x:c r="B7"/>
-      <x:c r="C7"/>
-      <x:c r="D7"/>
-      <x:c r="E7"/>
-      <x:c r="F7"/>
-      <x:c r="G7"/>
-      <x:c r="H7"/>
-      <x:c r="I7"/>
-      <x:c r="J7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8"/>
@@ -33041,9 +33680,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Ra9f0d4762c154750"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="Red14ec43976b413a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rdebae918f4f94596"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc3c8540323df46bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R89123a148bde41bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rbfb375263a4c4223"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -33080,7 +33719,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="119" t="str">
-        <x:v>실제 편집 가이드 3종 · 원본 스키마 고정형 V2</x:v>
+        <x:v>실제 편집 가이드 3종 · 원본 스키마 고정형 v5.4</x:v>
       </x:c>
       <x:c r="B1" s="31"/>
       <x:c r="C1" s="31"/>
@@ -33107,7 +33746,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="120" t="str">
-        <x:v>최초 템플릿 구조를 유지해 새 시트/새 열을 추가하지 않습니다. 5프레임 분석은 03의 action_pattern·timing_rule에 흡수하고, action_pattern은 동작·카메라·컷·효과·5프레임 근거까지 상세 기록합니다. personalization_rule은 새 사용자 영상에서 실제로 바꿀 수 있는 규칙만 정의하며, 레퍼런스 자막 문구는 고정 재사용하지 않고 LLM이 새 영상 내용에 맞춰 생성합니다.</x:v>
+        <x:v>최초 템플릿 구조를 유지해 새 시트·새 열을 추가하지 않습니다. 주술회전·동그리오의 업로드 JSON 근거를 action_pattern·timing_rule에 흡수하고, 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -34221,7 +34860,7 @@
         <x:v>HOOK_SETUP_A</x:v>
       </x:c>
       <x:c r="J19" s="69" t="str">
-        <x:v>[ACTION] 여성 정면 미디엄 구도. 오른손 손가락 포즈를 얼굴 옆에 고정하고 왼팔/손바닥을 카메라 전방으로 내민다. | [FRAME] 30fps F000-F009 (10f); phase=SETUP_EMPTY; shot=S1_WOMAN_DRINK | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left wrist/palm; camera position locked pre/post; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=SHOT_START@F000; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; next reveal anchor=F12; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F000-F004:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=오른손 손가락 포즈 + 왼손을 카메라 쪽으로 내민 상태; event=NONE; zoom=1; speed=1; MAD=1.572/4.418; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F005-F009:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=오른손 손가락 포즈 + 왼손을 카메라 쪽으로 내민 상태; event=NONE; zoom=1; speed=1; MAD=2.777/8.612; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 정면 미디엄 구도. 오른손 손가락 포즈를 얼굴 옆에 고정하고 왼팔/손바닥을 카메라 전방으로 내민다. | [FRAME] 30fps F000-F009 (10f); phase=SETUP_EMPTY; shot=S1_WOMAN_DRINK | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left wrist/palm; camera position locked pre/post; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=SHOT_START@F000; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; next reveal anchor=F12; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F000-F004:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=오른손 손가락 포즈 + 왼손을 카메라 쪽으로 내민 상태; event=NONE; zoom=1; speed=1; MAD=1.572/4.418; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F005-F009:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=오른손 손가락 포즈 + 왼손을 카메라 쪽으로 내민 상태; event=NONE; zoom=1; speed=1; MAD=2.777/8.612; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K19" s="69" t="str">
         <x:v>30fps; segment=F000-F009; start=0ms; end=333.333ms; duration=10f; event=SHOT_START@F000; hard_cut_in=-1; transition=NONE; transition_frames=0; speed=1; zoom=1; audio_anchor=NO_REQUIRED_EVENT; next reveal anchor=F12</x:v>
@@ -34248,7 +34887,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S19" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T19" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34319,7 +34958,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S20" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T20" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34390,7 +35029,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S21" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T21" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34434,7 +35073,7 @@
         <x:v>RESULT_HOLD_A</x:v>
       </x:c>
       <x:c r="J22" s="69" t="str">
-        <x:v>[ACTION] 상품을 카메라 가까운 전경에 유지하고 오른손 포즈·얼굴·카메라 위치를 크게 바꾸지 않는다. | [FRAME] 30fps F013-F058 (46f); phase=PRODUCT_HOLD; shot=S1_WOMAN_DRINK | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left wrist/palm; camera position locked pre/post; state=PRODUCT_A_LARGE_ICED_DRINK_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain source cadence until hard cut F59; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F010-F014:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=F10-11 FULL_FRAME_VERTICAL_MOTION_BLUR | F12 PRODUCT_A_REVEAL; zoom=1; speed=1; MAD=11.324/29.809; cmd=F10-11:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F12:MATCH_CUT_PRE_POST_TAKE+PRODUCT_A_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F015-F019:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.153/5.43; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F020-F024:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.002/5.201; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F025-F029:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.546/4.754; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F030-F034:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.648/4.412; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F035-F039:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.103/4.143; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F040-F044:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.903/3.612; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F045-F049:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.582/3.735; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F050-F054:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.165/3.814; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F055-F059:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=F59 HARD_CUT S1→S2; zoom=1; speed=1; MAD=14.665/69.427; cmd=F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 상품을 카메라 가까운 전경에 유지하고 오른손 포즈·얼굴·카메라 위치를 크게 바꾸지 않는다. | [FRAME] 30fps F013-F058 (46f); phase=PRODUCT_HOLD; shot=S1_WOMAN_DRINK | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left wrist/palm; camera position locked pre/post; state=PRODUCT_A_LARGE_ICED_DRINK_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain source cadence until hard cut F59; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F010-F014:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=F10-11 FULL_FRAME_VERTICAL_MOTION_BLUR | F12 PRODUCT_A_REVEAL; zoom=1; speed=1; MAD=11.324/29.809; cmd=F10-11:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F12:MATCH_CUT_PRE_POST_TAKE+PRODUCT_A_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F015-F019:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.153/5.43; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F020-F024:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.002/5.201; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F025-F029:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.546/4.754; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F030-F034:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.648/4.412; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F035-F039:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.103/4.143; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F040-F044:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.903/3.612; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F045-F049:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.582/3.735; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F050-F054:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=왼손으로 큰 아이스 음료를 전경에 제시하고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.165/3.814; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F055-F059:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=F59 HARD_CUT S1→S2; zoom=1; speed=1; MAD=14.665/69.427; cmd=F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K22" s="69" t="str">
         <x:v>30fps; segment=F013-F058; start=433.333ms; end=1966.667ms; duration=46f; event=HOLD@NONE; hard_cut_in=-1; transition=NONE; transition_frames=0; speed=1; zoom=1; audio_anchor=NO_REQUIRED_EVENT; maintain source cadence until hard cut F59; 5F_exact=F010-F014:F10-11:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F12:MATCH_CUT_PRE_POST_TAKE+PRODUCT_A_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F055-F059:F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -34461,7 +35100,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S22" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T22" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34499,13 +35138,13 @@
         <x:v>3666.667</x:v>
       </x:c>
       <x:c r="H23" s="69" t="str">
-        <x:v>S2 남성 팔 스윕 세팅</x:v>
+        <x:v>S2 팔 스윕 세팅</x:v>
       </x:c>
       <x:c r="I23" s="69" t="str">
         <x:v>HOOK_SETUP_B</x:v>
       </x:c>
       <x:c r="J23" s="69" t="str">
-        <x:v>[ACTION] F59 하드컷으로 검은 상의 남성 착석 구도 진입. 오른팔/손을 얼굴 앞에서 스윕하며 다른 팔은 옆/전방에 둔다. | [FRAME] 30fps F059-F109 (51f); phase=SETUP_EMPTY; shot=S2_MAN_RED_DRINK | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=sunglasses/face center + forearm/wrist line + seated torso; pre/post crop anchor locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F059; hard_cut_in=59; transition=HARD_CUT_S1_TO_S2/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F59 1.967s; nearest_beat=1.765s Δ+202ms; nearest_onset=1.974s Δ-7ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F055-F059:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=F59 HARD_CUT S1→S2; zoom=1; speed=1; MAD=14.665/69.427; cmd=F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F060-F064:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.206/2.417; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F065-F069:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.247/1.874; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F070-F074:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.216/2.115; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F075-F079:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.186/1.818; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F080-F084:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.691/3.743; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F085-F089:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=2.063/4.081; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F090-F094:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=3.685/5.734; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F095-F099:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=4.282/8.748; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F100-F104:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=6.276/11.329; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F105-F109:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=검은 상의 남성이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=6.69/13.234; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
+        <x:v>[ACTION] F59 하드컷으로 착석 구도 진입. 오른팔/손을 얼굴 앞에서 스윕하며 다른 팔은 옆/전방에 둔다. | [FRAME] 30fps F059-F109 (51f); phase=SETUP_EMPTY; shot=S2_MAN_RED_DRINK | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=sunglasses/face center + forearm/wrist line + seated torso; pre/post crop anchor locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F059; hard_cut_in=59; transition=HARD_CUT_S1_TO_S2/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F59 1.967s; nearest_beat=1.765s Δ+202ms; nearest_onset=1.974s Δ-7ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F055-F059:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=F59 HARD_CUT S1→S2; zoom=1; speed=1; MAD=14.665/69.427; cmd=F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F060-F064:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.206/2.417; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F065-F069:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.247/1.874; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F070-F074:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.216/2.115; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F075-F079:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.186/1.818; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F080-F084:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=1.691/3.743; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F085-F089:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=2.063/4.081; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F090-F094:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=3.685/5.734; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F095-F099:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=4.282/8.748; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F100-F104:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=6.276/11.329; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F105-F109:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 오른팔/손을 얼굴 앞에서 스윕하며 왼팔을 옆으로 유지; event=NONE; zoom=1; speed=1; MAD=6.69/13.234; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K23" s="69" t="str">
         <x:v>30fps; segment=F059-F109; start=1966.667ms; end=3666.667ms; duration=51f; event=HARD_CUT_IN@F059; hard_cut_in=59; transition=HARD_CUT_S1_TO_S2; transition_frames=0; speed=1; zoom=1; audio_anchor=F59 1.967s; nearest_beat=1.765s Δ+202ms; nearest_onset=1.974s Δ-7ms; 5F_exact=F055-F059:F59:HARD_CUT_TO_S2; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -34532,7 +35171,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S23" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T23" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34603,7 +35242,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S24" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T24" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34674,7 +35313,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S25" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T25" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34745,7 +35384,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S26" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T26" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34789,7 +35428,7 @@
         <x:v>RESULT_HOLD_B</x:v>
       </x:c>
       <x:c r="J27" s="69" t="str">
-        <x:v>[ACTION] 붉은 음료를 든 상태로 1.23배 펀치인 구도를 유지하고 손·얼굴 중심 구도를 안정적으로 보여준다. | [FRAME] 30fps F113-F158 (46f); phase=PRODUCT_HOLD_PUNCHIN; shot=S2_MAN_RED_DRINK | [CAMERA] framing=MEDIUM_CLOSE_DIGITAL_PUNCHIN; motion=DIGITAL_PUNCH_IN_HELD; zoom=1.23@(0.50,0.43) main-layer estimated visual center | [SUBJECT] match_anchor=sunglasses/face center + forearm/wrist line + seated torso; pre/post crop anchor locked; state=PRODUCT_B_RED_DRINK_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until hard cut F159; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F110-F114:PUNCH_IN_PRE_REVEAL→REVEAL_ZOOM_BLUR→PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=F110 DIGITAL_PUNCH_IN scale≈1.23 | F111 RADIAL/ZOOM_BLUR | F112 PRODUCT_B_REVEAL; zoom=1.23; speed=1; MAD=29.142/49.473; cmd=F110:ZOOM=1.23; F111:EFFECT=RADIAL_ZOOM_BLUR; F112:MATCH_CUT_PRE_POST_TAKE+PRODUCT_B_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F115-F119:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=6.409/9.653; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F120-F124:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.28/11.069; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F125-F129:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=7.224/11.779; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F130-F134:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=8.28/13.695; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F135-F139:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.35/7.466; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F140-F144:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.54/9.389; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F145-F149:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=8.998/13.009; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F150-F154:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.603/10.963; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F155-F159:PRODUCT_HOLD_PUNCH_IN→SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=F159 HARD_CUT S2→S3; zoom=1.23; speed=1; MAD=19.784/71.002; cmd=F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 붉은 음료를 든 상태로 1.23배 펀치인 구도를 유지하고 손·얼굴 중심 구도를 안정적으로 보여준다. | [FRAME] 30fps F113-F158 (46f); phase=PRODUCT_HOLD_PUNCHIN; shot=S2_MAN_RED_DRINK | [CAMERA] framing=MEDIUM_CLOSE_DIGITAL_PUNCHIN; motion=DIGITAL_PUNCH_IN_HELD; zoom=1.23@(0.50,0.43) main-layer estimated visual center | [SUBJECT] match_anchor=sunglasses/face center + forearm/wrist line + seated torso; pre/post crop anchor locked; state=PRODUCT_B_RED_DRINK_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until hard cut F159; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F110-F114:PUNCH_IN_PRE_REVEAL→REVEAL_ZOOM_BLUR→PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=F110 DIGITAL_PUNCH_IN scale≈1.23 | F111 RADIAL/ZOOM_BLUR | F112 PRODUCT_B_REVEAL; zoom=1.23; speed=1; MAD=29.142/49.473; cmd=F110:ZOOM=1.23; F111:EFFECT=RADIAL_ZOOM_BLUR; F112:MATCH_CUT_PRE_POST_TAKE+PRODUCT_B_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F115-F119:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=6.409/9.653; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F120-F124:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.28/11.069; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F125-F129:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=7.224/11.779; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F130-F134:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=8.28/13.695; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F135-F139:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.35/7.466; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F140-F144:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.54/9.389; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F145-F149:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=8.998/13.009; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F150-F154:PRODUCT_HOLD_PUNCH_IN/MEDIUM_CLOSE_PUNCHIN; action=붉은 음료를 얼굴 앞에 들고 펀치인 구도를 유지; event=NONE; zoom=1.23; speed=1; MAD=5.603/10.963; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F155-F159:PRODUCT_HOLD_PUNCH_IN→SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=F159 HARD_CUT S2→S3; zoom=1.23; speed=1; MAD=19.784/71.002; cmd=F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K27" s="69" t="str">
         <x:v>30fps; segment=F113-F158; start=3766.667ms; end=5300ms; duration=46f; event=HOLD@NONE; hard_cut_in=-1; transition=NONE; transition_frames=0; speed=1; zoom=1.23; audio_anchor=NO_REQUIRED_EVENT; maintain cadence until hard cut F159; 5F_exact=F110-F114:F110:ZOOM=1.23; F111:EFFECT=RADIAL_ZOOM_BLUR; F112:MATCH_CUT_PRE_POST_TAKE+PRODUCT_B_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F155-F159:F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -34816,7 +35455,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S27" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T27" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34854,13 +35493,13 @@
         <x:v>7000</x:v>
       </x:c>
       <x:c r="H28" s="69" t="str">
-        <x:v>S3 여성 손바닥 세팅</x:v>
+        <x:v>S3 손바닥 세팅</x:v>
       </x:c>
       <x:c r="I28" s="69" t="str">
         <x:v>HOOK_SETUP_C</x:v>
       </x:c>
       <x:c r="J28" s="69" t="str">
-        <x:v>[ACTION] F159 하드컷으로 여성 정면 구도 진입. 오른손 손가락 포즈를 고정하고 왼손 손바닥을 카메라 쪽으로 펼친다. | [FRAME] 30fps F159-F209 (51f); phase=SETUP_EMPTY; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F159; hard_cut_in=159; transition=HARD_CUT_S2_TO_S3/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F159 5.300s; nearest_beat=5.224s Δ+76ms; nearest_onset=5.642s Δ-342ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F155-F159:PRODUCT_HOLD_PUNCH_IN→SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=F159 HARD_CUT S2→S3; zoom=1.23; speed=1; MAD=19.784/71.002; cmd=F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F160-F164:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.079/4.478; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F165-F169:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.068/4.288; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F170-F174:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.047/4.347; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F175-F179:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.942/3.899; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F180-F184:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.689/4.055; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F185-F189:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.934/3.817; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F190-F194:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=3.047/7.97; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F195-F199:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=3.057/6.204; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F200-F204:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.878/4.114; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F205-F209:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=여성이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=5.46/21.06; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
+        <x:v>[ACTION] F159 하드컷으로 정면 구도 진입. 오른손 손가락 포즈를 고정하고 왼손 손바닥을 카메라 쪽으로 펼친다. | [FRAME] 30fps F159-F209 (51f); phase=SETUP_EMPTY; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F159; hard_cut_in=159; transition=HARD_CUT_S2_TO_S3/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F159 5.300s; nearest_beat=5.224s Δ+76ms; nearest_onset=5.642s Δ-342ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F155-F159:PRODUCT_HOLD_PUNCH_IN→SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=F159 HARD_CUT S2→S3; zoom=1.23; speed=1; MAD=19.784/71.002; cmd=F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F160-F164:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.079/4.478; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F165-F169:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.068/4.288; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F170-F174:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=2.047/4.347; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F175-F179:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.942/3.899; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F180-F184:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.689/4.055; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F185-F189:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.934/3.817; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F190-F194:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=3.047/7.97; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F195-F199:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=3.057/6.204; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F200-F204:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=1.878/4.114; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F205-F209:SETUP_EMPTY/MEDIUM_PORTRAIT_FRONT; action=인물이 오른손 손가락 포즈 + 왼손 손바닥을 전경에 펼침; event=NONE; zoom=1; speed=1; MAD=5.46/21.06; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K28" s="69" t="str">
         <x:v>30fps; segment=F159-F209; start=5300ms; end=7000ms; duration=51f; event=HARD_CUT_IN@F159; hard_cut_in=159; transition=HARD_CUT_S2_TO_S3; transition_frames=0; speed=1; zoom=1; audio_anchor=F159 5.300s; nearest_beat=5.224s Δ+76ms; nearest_onset=5.642s Δ-342ms; 5F_exact=F155-F159:F159:HARD_CUT_TO_S3; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -34887,7 +35526,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S28" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T28" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34931,7 +35570,7 @@
         <x:v>TRANSITION_C</x:v>
       </x:c>
       <x:c r="J29" s="69" t="str">
-        <x:v>[ACTION] 메인 영상만 수직 방향 전 프레임 블러로 2프레임 가리고, 상단 PIP는 선명하게 유지한다. | [FRAME] 30fps F210-F211 (2f); phase=REVEAL_BLUR; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=EMPTY→PRODUCT_C_PENDING | [EDIT] type=MOTION_BLUR@F210; hard_cut_in=-1; transition=FULL_FRAME_VERTICAL_MOTION_BLUR_ON_MAIN/2f; blur=F210-211 vertical full-frame motion blur; instant clear F212; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 메인 영상만 수직 방향 전 프레임 블러로 2프레임 가리고, 상단 PIP는 선명하게 유지한다. | [FRAME] 30fps F210-F211 (2f); phase=REVEAL_BLUR; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=EMPTY→PRODUCT_C_PENDING | [EDIT] type=MOTION_BLUR@F210; hard_cut_in=-1; transition=FULL_FRAME_VERTICAL_MOTION_BLUR_ON_MAIN/2f; blur=F210-211 vertical full-frame motion blur; instant clear F212; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K29" s="69" t="str">
         <x:v>30fps; segment=F210-F211; start=7000ms; end=7066.667ms; duration=2f; event=MOTION_BLUR@F210; hard_cut_in=-1; transition=FULL_FRAME_VERTICAL_MOTION_BLUR_ON_MAIN; transition_frames=2; speed=1; zoom=1; audio_anchor=F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; 5F_exact=F210-F214:F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -34958,7 +35597,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S29" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T29" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -34996,13 +35635,13 @@
         <x:v>7100</x:v>
       </x:c>
       <x:c r="H30" s="69" t="str">
-        <x:v>S3 케이크 정확 등장 프레임</x:v>
+        <x:v>S3 디저트 정확 등장 프레임</x:v>
       </x:c>
       <x:c r="I30" s="69" t="str">
         <x:v>REVEAL_C</x:v>
       </x:c>
       <x:c r="J30" s="69" t="str">
-        <x:v>[ACTION] 동일 구도의 상품 있음 후테이크로 매치컷해 케이크 접시를 화면 하단/전경에 즉시 등장시킨다. | [FRAME] 30fps F212-F212 (1f); phase=PRODUCT_REVEAL; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=PRODUCT_C_CAKE_VISIBLE | [EDIT] type=MATCH_CUT_REVEAL@F212; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE/0f; blur=NONE; blur clears on reveal; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC | [SHAKE] OPTIONAL_REUSABLE_SHAKE(trigger=semantic impact/reveal/beat accent only; default=OFF; duration=3-5f; translate_x/y=±1.5~2.5% frame; rotate=±0.5~0.8deg; scale=1.02; alternate direction then damp to 0; never continuous; disable if readability/stability degrades)</x:v>
+        <x:v>[ACTION] 동일 구도의 상품 있음 후테이크로 매치컷해 디저트 접시를 화면 하단/전경에 즉시 등장시킨다. | [FRAME] 30fps F212-F212 (1f); phase=PRODUCT_REVEAL; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=PRODUCT_C_CAKE_VISIBLE | [EDIT] type=MATCH_CUT_REVEAL@F212; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE/0f; blur=NONE; blur clears on reveal; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC | [SHAKE] OPTIONAL_REUSABLE_SHAKE(trigger=semantic impact/reveal/beat accent only; default=OFF; duration=3-5f; translate_x/y=±1.5~2.5% frame; rotate=±0.5~0.8deg; scale=1.02; alternate direction then damp to 0; never continuous; disable if readability/stability degrades)</x:v>
       </x:c>
       <x:c r="K30" s="69" t="str">
         <x:v>30fps; segment=F212-F212; start=7066.667ms; end=7100ms; duration=1f; event=MATCH_CUT_REVEAL@F212; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE; transition_frames=0; speed=1; zoom=1; audio_anchor=F212 7.067s; nearest_beat=6.873s Δ+194ms; nearest_onset=7.082s Δ-15ms; 5F_exact=F210-F214:F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35029,7 +35668,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S30" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T30" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -35067,13 +35706,13 @@
         <x:v>8733.333</x:v>
       </x:c>
       <x:c r="H31" s="69" t="str">
-        <x:v>S3 케이크 결과 홀드</x:v>
+        <x:v>S3 디저트 결과 홀드</x:v>
       </x:c>
       <x:c r="I31" s="69" t="str">
         <x:v>RESULT_HOLD_C</x:v>
       </x:c>
       <x:c r="J31" s="69" t="str">
-        <x:v>[ACTION] 케이크 접시를 전경에 든 상태로 오른손 포즈·얼굴·카메라 프레이밍을 안정적으로 유지한다. | [FRAME] 30fps F213-F261 (49f); phase=PRODUCT_HOLD; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=PRODUCT_C_CAKE_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until hard cut F262; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F215-F219:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=5.596/8.99; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F220-F224:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=4.285/8.324; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F225-F229:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.499/8.36; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F230-F234:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=4.467/6.866; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F235-F239:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.064/4.057; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F240-F244:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.009/5.206; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F245-F249:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.168/4.929; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F250-F254:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.592/7.268; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F255-F259:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=케이크 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.479/2.88; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F260-F264:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=F262 HARD_CUT S3→S4; zoom=1; speed=1; MAD=12.854/62.473; cmd=F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 디저트 접시를 전경에 든 상태로 오른손 포즈·얼굴·카메라 프레이밍을 안정적으로 유지한다. | [FRAME] 30fps F213-F261 (49f); phase=PRODUCT_HOLD; shot=S3_WOMAN_CAKE | [CAMERA] framing=MEDIUM_PORTRAIT_FRONT; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=face/head center + right-hand finger gesture + left open-palm/wrist; camera locked; state=PRODUCT_C_CAKE_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until hard cut F262; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F210-F214:REVEAL_BLUR→PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=F210-211 FULL_FRAME_VERTICAL_MOTION_BLUR | F212 PRODUCT_C_REVEAL; zoom=1; speed=1; MAD=12.827/33.229; cmd=F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F215-F219:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=5.596/8.99; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F220-F224:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=4.285/8.324; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F225-F229:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.499/8.36; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F230-F234:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=4.467/6.866; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F235-F239:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.064/4.057; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F240-F244:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.009/5.206; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F245-F249:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=3.168/4.929; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F250-F254:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=2.592/7.268; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F255-F259:PRODUCT_HOLD/MEDIUM_PORTRAIT_FRONT; action=디저트 접시를 전경에 들고 오른손 포즈 유지; event=NONE; zoom=1; speed=1; MAD=1.479/2.88; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F260-F264:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=F262 HARD_CUT S3→S4; zoom=1; speed=1; MAD=12.854/62.473; cmd=F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K31" s="69" t="str">
         <x:v>30fps; segment=F213-F261; start=7100ms; end=8733.333ms; duration=49f; event=HOLD@NONE; hard_cut_in=-1; transition=NONE; transition_frames=0; speed=1; zoom=1; audio_anchor=NO_REQUIRED_EVENT; maintain cadence until hard cut F262; 5F_exact=F210-F214:F210-211:EFFECT=FULL_FRAME_VERTICAL_MOTION_BLUR; F212:MATCH_CUT_PRE_POST_TAKE+PRODUCT_C_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F260-F264:F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35100,7 +35739,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S31" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T31" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -35138,13 +35777,13 @@
         <x:v>10300</x:v>
       </x:c>
       <x:c r="H32" s="69" t="str">
-        <x:v>S4 남성 양손 제스처 세팅</x:v>
+        <x:v>S4 양손 제스처 세팅</x:v>
       </x:c>
       <x:c r="I32" s="69" t="str">
         <x:v>HOOK_SETUP_D</x:v>
       </x:c>
       <x:c r="J32" s="69" t="str">
-        <x:v>[ACTION] F262 하드컷으로 남성 착석 구도 진입. 두 손을 겹치거나 모아 카메라 전방으로 밀며 공개 동작을 준비한다. | [FRAME] 30fps F262-F308 (47f); phase=SETUP_EMPTY; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F262; hard_cut_in=262; transition=HARD_CUT_S3_TO_S4/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F262 8.733s; nearest_beat=8.545s Δ+188ms; nearest_onset=8.638s Δ+95ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F260-F264:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=F262 HARD_CUT S3→S4; zoom=1; speed=1; MAD=12.854/62.473; cmd=F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F265-F269:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=0.455/0.887; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F270-F274:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=0.947/1.503; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F275-F279:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=1.578/3.511; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F280-F284:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=2.576/4.436; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F285-F289:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=3.712/5.152; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F290-F294:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=3.29/8.329; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F295-F299:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=6.352/9.039; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F300-F304:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=남성이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=4.569/9.056; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F305-F309:SETUP_EMPTY→REVEAL_PROGRESSIVE_BLUR/MEDIUM_WIDE_SEATED; action=손이 펴지는 순간 진행성 블러로 전환; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR; zoom=1; speed=1; MAD=7.43/21.505; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] F262 하드컷으로 착석 구도 진입. 두 손을 겹치거나 모아 카메라 전방으로 밀며 공개 동작을 준비한다. | [FRAME] 30fps F262-F308 (47f); phase=SETUP_EMPTY; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=EMPTY_OR_NOT_YET_VISIBLE | [EDIT] type=HARD_CUT_IN@F262; hard_cut_in=262; transition=HARD_CUT_S3_TO_S4/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F262 8.733s; nearest_beat=8.545s Δ+188ms; nearest_onset=8.638s Δ+95ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F260-F264:PRODUCT_HOLD→SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=F262 HARD_CUT S3→S4; zoom=1; speed=1; MAD=12.854/62.473; cmd=F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F265-F269:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=0.455/0.887; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F270-F274:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=0.947/1.503; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F275-F279:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=1.578/3.511; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F280-F284:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=2.576/4.436; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F285-F289:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=3.712/5.152; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F290-F294:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=3.29/8.329; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F295-F299:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=6.352/9.039; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F300-F304:SETUP_EMPTY/MEDIUM_WIDE_SEATED; action=인물이 두 손을 겹쳐/모아 전방으로 밀어내는 동작; event=NONE; zoom=1; speed=1; MAD=4.569/9.056; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F305-F309:SETUP_EMPTY→REVEAL_PROGRESSIVE_BLUR/MEDIUM_WIDE_SEATED; action=손이 펴지는 순간 진행성 블러로 전환; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR; zoom=1; speed=1; MAD=7.43/21.505; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K32" s="69" t="str">
         <x:v>30fps; segment=F262-F308; start=8733.333ms; end=10300ms; duration=47f; event=HARD_CUT_IN@F262; hard_cut_in=262; transition=HARD_CUT_S3_TO_S4; transition_frames=0; speed=1; zoom=1; audio_anchor=F262 8.733s; nearest_beat=8.545s Δ+188ms; nearest_onset=8.638s Δ+95ms; 5F_exact=F260-F264:F262:HARD_CUT_TO_S4; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F305-F309:F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35171,7 +35810,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S32" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T32" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -35215,7 +35854,7 @@
         <x:v>TRANSITION_D</x:v>
       </x:c>
       <x:c r="J33" s="69" t="str">
-        <x:v>[ACTION] F309에서 블러를 시작하고 F310-311에서 강도를 높여 손이 펼쳐지는 순간과 상품 교체를 가린다. PIP는 영향받지 않는다. | [FRAME] 30fps F309-F311 (3f); phase=PROGRESSIVE_REVEAL_BLUR; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=EMPTY→PRODUCT_D_PENDING | [EDIT] type=PROGRESSIVE_MOTION_BLUR@F309; hard_cut_in=-1; transition=PROGRESSIVE_FULL_FRAME_BLUR_ON_MAIN/3f; blur=F309 mild blur → F310-311 strong full-frame blur; clear at F312; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F309 10.300s nearest_onset=10.310s Δ-10ms; F312 10.400s nearest_onset=10.310s Δ+90ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F305-F309:SETUP_EMPTY→REVEAL_PROGRESSIVE_BLUR/MEDIUM_WIDE_SEATED; action=손이 펴지는 순간 진행성 블러로 전환; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR; zoom=1; speed=1; MAD=7.43/21.505; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] F309에서 블러를 시작하고 F310-311에서 강도를 높여 손이 펼쳐지는 순간과 상품 교체를 가린다. PIP는 영향받지 않는다. | [FRAME] 30fps F309-F311 (3f); phase=PROGRESSIVE_REVEAL_BLUR; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=EMPTY→PRODUCT_D_PENDING | [EDIT] type=PROGRESSIVE_MOTION_BLUR@F309; hard_cut_in=-1; transition=PROGRESSIVE_FULL_FRAME_BLUR_ON_MAIN/3f; blur=F309 mild blur → F310-311 strong full-frame blur; clear at F312; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F309 10.300s nearest_onset=10.310s Δ-10ms; F312 10.400s nearest_onset=10.310s Δ+90ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F305-F309:SETUP_EMPTY→REVEAL_PROGRESSIVE_BLUR/MEDIUM_WIDE_SEATED; action=손이 펴지는 순간 진행성 블러로 전환; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR; zoom=1; speed=1; MAD=7.43/21.505; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K33" s="69" t="str">
         <x:v>30fps; segment=F309-F311; start=10300ms; end=10400ms; duration=3f; event=PROGRESSIVE_MOTION_BLUR@F309; hard_cut_in=-1; transition=PROGRESSIVE_FULL_FRAME_BLUR_ON_MAIN; transition_frames=3; speed=1; zoom=1; audio_anchor=F309 10.300s nearest_onset=10.310s Δ-10ms; F312 10.400s nearest_onset=10.310s Δ+90ms; 5F_exact=F305-F309:F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F310-F314:F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35242,7 +35881,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S33" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T33" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -35280,13 +35919,13 @@
         <x:v>10433.333</x:v>
       </x:c>
       <x:c r="H34" s="69" t="str">
-        <x:v>S4 빵/페이스트리 정확 등장 프레임</x:v>
+        <x:v>S4 베이커리 메뉴 정확 등장 프레임</x:v>
       </x:c>
       <x:c r="I34" s="69" t="str">
         <x:v>REVEAL_D</x:v>
       </x:c>
       <x:c r="J34" s="69" t="str">
-        <x:v>[ACTION] 동일 구도의 후테이크로 매치컷해 빵/페이스트리 접시를 손 아래 전경에 즉시 등장시킨다. | [FRAME] 30fps F312-F312 (1f); phase=PRODUCT_REVEAL; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=PRODUCT_D_PASTRY_VISIBLE | [EDIT] type=MATCH_CUT_REVEAL@F312; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE/0f; blur=NONE; progressive blur clears on reveal; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F312 10.400s; nearest_beat=10.194s Δ+206ms; nearest_onset=10.310s Δ+90ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC | [SHAKE] OPTIONAL_REUSABLE_SHAKE(trigger=semantic impact/reveal/beat accent only; default=OFF; duration=3-5f; translate_x/y=±1.5~2.5% frame; rotate=±0.5~0.8deg; scale=1.02; alternate direction then damp to 0; never continuous; disable if readability/stability degrades)</x:v>
+        <x:v>[ACTION] 동일 구도의 후테이크로 매치컷해 베이커리 메뉴 접시를 손 아래 전경에 즉시 등장시킨다. | [FRAME] 30fps F312-F312 (1f); phase=PRODUCT_REVEAL; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=PRODUCT_D_PASTRY_VISIBLE | [EDIT] type=MATCH_CUT_REVEAL@F312; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE/0f; blur=NONE; progressive blur clears on reveal; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] F312 10.400s; nearest_beat=10.194s Δ+206ms; nearest_onset=10.310s Δ+90ms; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC | [SHAKE] OPTIONAL_REUSABLE_SHAKE(trigger=semantic impact/reveal/beat accent only; default=OFF; duration=3-5f; translate_x/y=±1.5~2.5% frame; rotate=±0.5~0.8deg; scale=1.02; alternate direction then damp to 0; never continuous; disable if readability/stability degrades)</x:v>
       </x:c>
       <x:c r="K34" s="69" t="str">
         <x:v>30fps; segment=F312-F312; start=10400ms; end=10433.333ms; duration=1f; event=MATCH_CUT_REVEAL@F312; hard_cut_in=-1; transition=MATCH_CUT_PRE_POST_TAKE; transition_frames=0; speed=1; zoom=1; audio_anchor=F312 10.400s; nearest_beat=10.194s Δ+206ms; nearest_onset=10.310s Δ+90ms; 5F_exact=F310-F314:F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35313,7 +35952,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S34" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T34" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -35351,13 +35990,13 @@
         <x:v>12066.667</x:v>
       </x:c>
       <x:c r="H35" s="69" t="str">
-        <x:v>S4 빵/페이스트리 결과 홀드</x:v>
+        <x:v>S4 베이커리 메뉴 결과 홀드</x:v>
       </x:c>
       <x:c r="I35" s="69" t="str">
         <x:v>RESULT_HOLD_D</x:v>
       </x:c>
       <x:c r="J35" s="69" t="str">
-        <x:v>[ACTION] 접시와 상품을 화면 하단/전경에 유지하면서 펼친 손과 얼굴 구도를 안정적으로 보여준다. | [FRAME] 30fps F313-F361 (49f); phase=PRODUCT_HOLD; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=PRODUCT_D_PASTRY_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until loop hard cut F362; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F315-F319:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=6.234/8.559; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F320-F324:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=5.232/9.415; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F325-F329:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.612/9.288; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F330-F334:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.779/6.466; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F335-F339:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.551/5.853; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F340-F344:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.858/5.812; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F345-F349:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.174/5.257; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F350-F354:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.829/5.293; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F355-F359:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=빵/페이스트리 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.927/5.128; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F360-F364:PRODUCT_HOLD→LOOP_RESET_SETUP/MEDIUM_PORTRAIT_FRONT_LOOP; action=첫 장면 빈손 포즈로 루프 재시작; event=F362 HARD_CUT/LOOP_RESET S4→S1; zoom=1; speed=1; MAD=14.489/65.692; cmd=F362:HARD_CUT_LOOP_RESET_TO_S1; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
+        <x:v>[ACTION] 접시와 상품을 화면 하단/전경에 유지하면서 펼친 손과 얼굴 구도를 안정적으로 보여준다. | [FRAME] 30fps F313-F361 (49f); phase=PRODUCT_HOLD; shot=S4_MAN_PASTRY | [CAMERA] framing=MEDIUM_WIDE_SEATED; motion=STATIC_FIXED_PHONE; zoom=1@(0.50,0.50) canvas center; no digital zoom | [SUBJECT] match_anchor=head center + both wrist/hand centerline + seated torso; camera locked; state=PRODUCT_D_PASTRY_VISIBLE | [EDIT] type=HOLD@NO_SINGLE_EVENT; hard_cut_in=-1; transition=NONE/0f; blur=NONE; scope=MAIN_VIDEO_ONLY_FOR_ZOOM_BLUR; PIP_EXCLUDED_FROM_MAIN_EFFECTS; layer=MAIN_VIDEO_BASE → MAIN_LAYER_EFFECTS → VIDEO_PIP_TOP | [PIP] bbox=(0.118,0.000,0.444,0.140); behavior=PERSISTENT; SCREEN_FIXED; OPAQUE; NO_BORDER; source-synced VIDEO_PIP; main-layer zoom/blur does not transform PIP | [AUDIO_COLOR] NO_REQUIRED_EVENT; maintain cadence until loop hard cut F362; KEEP_SOURCE_COLOR; no per-cut LUT/grade; maintain exposure/WB continuity | [5F] F310-F314:REVEAL_PROGRESSIVE_BLUR→PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=F309-311 PROGRESSIVE_FULL_FRAME_BLUR | F312 PRODUCT_D_REVEAL; zoom=1; speed=1; MAD=16.702/29.721; cmd=F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F315-F319:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=6.234/8.559; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F320-F324:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=5.232/9.415; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F325-F329:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.612/9.288; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F330-F334:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.779/6.466; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F335-F339:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.551/5.853; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F340-F344:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=3.858/5.812; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F345-F349:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.174/5.257; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F350-F354:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.829/5.293; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F355-F359:PRODUCT_HOLD/MEDIUM_WIDE_SEATED; action=베이커리 메뉴 접시를 전경에 들고 손을 펼친 자세 유지; event=NONE; zoom=1; speed=1; MAD=2.927/5.128; cmd=KEEP_SHOT; speed=1.0; cut=NONE; transition=NONE; text_overlay=NONE; color=KEEP_SOURCE; PIP=SYNC || F360-F364:PRODUCT_HOLD→LOOP_RESET_SETUP/MEDIUM_PORTRAIT_FRONT_LOOP; action=첫 장면 빈손 포즈로 루프 재시작; event=F362 HARD_CUT/LOOP_RESET S4→S1; zoom=1; speed=1; MAD=14.489/65.692; cmd=F362:HARD_CUT_LOOP_RESET_TO_S1; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
       </x:c>
       <x:c r="K35" s="69" t="str">
         <x:v>30fps; segment=F313-F361; start=10433.333ms; end=12066.667ms; duration=49f; event=HOLD@NONE; hard_cut_in=-1; transition=NONE; transition_frames=0; speed=1; zoom=1; audio_anchor=NO_REQUIRED_EVENT; maintain cadence until loop hard cut F362; 5F_exact=F310-F314:F309-311:EFFECT=PROGRESSIVE_FULL_FRAME_BLUR; F312:MATCH_CUT_PRE_POST_TAKE+PRODUCT_D_VISIBLE; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC || F360-F364:F362:HARD_CUT_LOOP_RESET_TO_S1; speed=1.0; dissolve=0; fade=0; text_overlay=NONE; PIP=SYNC</x:v>
@@ -35384,7 +36023,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="S35" s="69" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>SUPERSEDED</x:v>
       </x:c>
       <x:c r="T35" s="69" t="str">
         <x:v>'12_SOURCE_GUIDES'!$G$847:$G$870</x:v>
@@ -37033,379 +37672,1043 @@
       </x:c>
     </x:row>
     <x:row r="59" ht="78" customHeight="1">
-      <x:c r="A59"/>
-      <x:c r="B59"/>
-      <x:c r="C59"/>
-      <x:c r="D59"/>
-      <x:c r="E59"/>
-      <x:c r="F59"/>
-      <x:c r="G59"/>
-      <x:c r="H59"/>
-      <x:c r="I59"/>
-      <x:c r="J59"/>
-      <x:c r="K59"/>
+      <x:c r="A59" t="str">
+        <x:v>gts_jujutsu_v5_01</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D59" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E59" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G59" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>인물 A 빈손 포즈 훅</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>HOOK_SETUP</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>인물 A가 고정 미디엄 구도에서 빈손 시그니처 포즈에 진입해 안정적으로 유지</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>POSE_HOLD_END_ANCHORED; S02와 신체·손·배경 특징점을 정렬하고 1500ms SFX 직전에 종료</x:v>
+      </x:c>
       <x:c r="L59"/>
-      <x:c r="M59"/>
-      <x:c r="N59"/>
-      <x:c r="O59"/>
-      <x:c r="P59"/>
-      <x:c r="Q59"/>
-      <x:c r="R59"/>
-      <x:c r="S59"/>
-      <x:c r="T59"/>
-      <x:c r="U59"/>
-      <x:c r="V59"/>
-      <x:c r="W59"/>
+      <x:c r="M59" t="str">
+        <x:v>promo.primary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>첫 공개 아이템은 실제 대표 메뉴/상품으로 정하고 동일 인물·구도·배경의 S02와 한 쌍으로 촬영</x:v>
+      </x:c>
+      <x:c r="O59" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P59" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q59" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R59" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S59" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T59" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U59" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V59" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W59" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="78" customHeight="1">
-      <x:c r="A60"/>
-      <x:c r="B60"/>
-      <x:c r="C60"/>
-      <x:c r="D60"/>
-      <x:c r="E60"/>
-      <x:c r="F60"/>
-      <x:c r="G60"/>
-      <x:c r="H60"/>
-      <x:c r="I60"/>
-      <x:c r="J60"/>
-      <x:c r="K60"/>
+      <x:c r="A60" t="str">
+        <x:v>gts_jujutsu_v5_02</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D60" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E60" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F60" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="G60" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>인물 A 첫 아이템 공개</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>MAGIC_REVEAL</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>S01과 동일 포즈·구도에서 인물 A의 손에 실제 음료가 나타난 상태로 시작해 결과를 유지</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>1500ms SFX 타격점 HARD_CUT_MATCH; speed=1.0; 디졸브·페이드 금지</x:v>
+      </x:c>
       <x:c r="L60"/>
-      <x:c r="M60"/>
-      <x:c r="N60"/>
-      <x:c r="O60"/>
-      <x:c r="P60"/>
-      <x:c r="Q60"/>
-      <x:c r="R60"/>
-      <x:c r="S60"/>
-      <x:c r="T60"/>
-      <x:c r="U60"/>
-      <x:c r="V60"/>
-      <x:c r="W60"/>
+      <x:c r="M60" t="str">
+        <x:v>promo.primary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>S01 마지막 프레임과 가장 일치하는 ITEM_PRESENT 프레임을 선택하고 실제 음료/상품만 노출</x:v>
+      </x:c>
+      <x:c r="O60" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P60" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q60" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R60" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S60" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T60" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U60" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V60" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W60" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="78" customHeight="1">
-      <x:c r="A61"/>
-      <x:c r="B61"/>
-      <x:c r="C61"/>
-      <x:c r="D61"/>
-      <x:c r="E61"/>
-      <x:c r="F61"/>
-      <x:c r="G61"/>
-      <x:c r="H61"/>
-      <x:c r="I61"/>
-      <x:c r="J61"/>
-      <x:c r="K61"/>
+      <x:c r="A61" t="str">
+        <x:v>gts_jujutsu_v5_03</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D61" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E61" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F61" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="G61" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>인물 B 빈손 포즈 셋업</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>SETUP</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>인물 B가 같은 고정 카메라에서 새로운 빈손 포즈를 취하고 안정 구간을 유지</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>POSE_HOLD_END_ANCHORED; S04와 포즈·배경을 정렬하고 5000ms SFX 직전에 종료</x:v>
+      </x:c>
       <x:c r="L61"/>
-      <x:c r="M61"/>
-      <x:c r="N61"/>
-      <x:c r="O61"/>
-      <x:c r="P61"/>
-      <x:c r="Q61"/>
-      <x:c r="R61"/>
-      <x:c r="S61"/>
-      <x:c r="T61"/>
-      <x:c r="U61"/>
-      <x:c r="V61"/>
-      <x:c r="W61"/>
+      <x:c r="M61" t="str">
+        <x:v>promo.secondary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>두 번째 출연자와 보조 메뉴를 사용하되 S04와 동일 인물·의상·배경 유지</x:v>
+      </x:c>
+      <x:c r="O61" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P61" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q61" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R61" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S61" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T61" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U61" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V61" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W61" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="78" customHeight="1">
-      <x:c r="A62"/>
-      <x:c r="B62"/>
-      <x:c r="C62"/>
-      <x:c r="D62"/>
-      <x:c r="E62"/>
-      <x:c r="F62"/>
-      <x:c r="G62"/>
-      <x:c r="H62"/>
-      <x:c r="I62"/>
-      <x:c r="J62"/>
-      <x:c r="K62"/>
+      <x:c r="A62" t="str">
+        <x:v>gts_jujutsu_v5_04</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F62" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="G62" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>인물 B 두 번째 아이템 공개</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>MAGIC_REVEAL</x:v>
+      </x:c>
+      <x:c r="J62" t="str">
+        <x:v>S03과 동일 포즈·구도에서 인물 B의 손에 다른 음료가 나타난 상태로 전환</x:v>
+      </x:c>
+      <x:c r="K62" t="str">
+        <x:v>5000ms SFX 타격점 HARD_CUT_MATCH; speed=1.0; 7000ms HARD_CUT</x:v>
+      </x:c>
       <x:c r="L62"/>
-      <x:c r="M62"/>
-      <x:c r="N62"/>
-      <x:c r="O62"/>
-      <x:c r="P62"/>
-      <x:c r="Q62"/>
-      <x:c r="R62"/>
-      <x:c r="S62"/>
-      <x:c r="T62"/>
-      <x:c r="U62"/>
-      <x:c r="V62"/>
-      <x:c r="W62"/>
+      <x:c r="M62" t="str">
+        <x:v>promo.secondary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N62" t="str">
+        <x:v>S03 마지막 프레임과 가장 일치하는 ITEM_PRESENT 프레임을 시작점으로 선택</x:v>
+      </x:c>
+      <x:c r="O62" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P62" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q62" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R62" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S62" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T62" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U62" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V62" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W62" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="78" customHeight="1">
-      <x:c r="A63"/>
-      <x:c r="B63"/>
-      <x:c r="C63"/>
-      <x:c r="D63"/>
-      <x:c r="E63"/>
-      <x:c r="F63"/>
-      <x:c r="G63"/>
-      <x:c r="H63"/>
-      <x:c r="I63"/>
-      <x:c r="J63"/>
-      <x:c r="K63"/>
+      <x:c r="A63" t="str">
+        <x:v>gts_jujutsu_v5_05</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D63" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E63" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F63" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="G63" t="n">
+        <x:v>8500</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>인물 A 새 빈손 포즈 셋업</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>SETUP</x:v>
+      </x:c>
+      <x:c r="J63" t="str">
+        <x:v>인물 A가 다시 등장해 제품 공개 전 새 빈손 포즈를 안정적으로 유지</x:v>
+      </x:c>
+      <x:c r="K63" t="str">
+        <x:v>POSE_HOLD_END_ANCHORED; S06과 정렬하고 8500ms SFX 직전에 종료</x:v>
+      </x:c>
       <x:c r="L63"/>
-      <x:c r="M63"/>
-      <x:c r="N63"/>
-      <x:c r="O63"/>
-      <x:c r="P63"/>
-      <x:c r="Q63"/>
-      <x:c r="R63"/>
-      <x:c r="S63"/>
-      <x:c r="T63"/>
-      <x:c r="U63"/>
-      <x:c r="V63"/>
-      <x:c r="W63"/>
+      <x:c r="M63" t="str">
+        <x:v>promo.tertiary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N63" t="str">
+        <x:v>세 번째 실제 메뉴의 형태를 고려해 손과 테이블이 가리지 않는 포즈 선택</x:v>
+      </x:c>
+      <x:c r="O63" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P63" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q63" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R63" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S63" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T63" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U63" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V63" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W63" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="78" customHeight="1">
-      <x:c r="A64"/>
-      <x:c r="B64"/>
-      <x:c r="C64"/>
-      <x:c r="D64"/>
-      <x:c r="E64"/>
-      <x:c r="F64"/>
-      <x:c r="G64"/>
-      <x:c r="H64"/>
-      <x:c r="I64"/>
-      <x:c r="J64"/>
-      <x:c r="K64"/>
+      <x:c r="A64" t="str">
+        <x:v>gts_jujutsu_v5_06</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D64" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E64" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F64" t="n">
+        <x:v>8500</x:v>
+      </x:c>
+      <x:c r="G64" t="n">
+        <x:v>10500</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>인물 A 제품 공개</x:v>
+      </x:c>
+      <x:c r="I64" t="str">
+        <x:v>MAGIC_REVEAL</x:v>
+      </x:c>
+      <x:c r="J64" t="str">
+        <x:v>S05와 동일 포즈·구도에서 인물 A가 실제 제품을 든 상태로 시작</x:v>
+      </x:c>
+      <x:c r="K64" t="str">
+        <x:v>8500ms SFX 타격점 HARD_CUT_MATCH; speed=1.0; 아이템 전체가 보이는 결과 홀드</x:v>
+      </x:c>
       <x:c r="L64"/>
-      <x:c r="M64"/>
-      <x:c r="N64"/>
-      <x:c r="O64"/>
-      <x:c r="P64"/>
-      <x:c r="Q64"/>
-      <x:c r="R64"/>
-      <x:c r="S64"/>
-      <x:c r="T64"/>
-      <x:c r="U64"/>
-      <x:c r="V64"/>
-      <x:c r="W64"/>
+      <x:c r="M64" t="str">
+        <x:v>promo.tertiary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N64" t="str">
+        <x:v>실제 촬영된 제품/대표 상품으로 치환하고 S05 경계의 포즈 일치 우선</x:v>
+      </x:c>
+      <x:c r="O64" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P64" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q64" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R64" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S64" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T64" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U64" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V64" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W64" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="78" customHeight="1">
-      <x:c r="A65"/>
-      <x:c r="B65"/>
-      <x:c r="C65"/>
-      <x:c r="D65"/>
-      <x:c r="E65"/>
-      <x:c r="F65"/>
-      <x:c r="G65"/>
-      <x:c r="H65"/>
-      <x:c r="I65"/>
-      <x:c r="J65"/>
-      <x:c r="K65"/>
+      <x:c r="A65" t="str">
+        <x:v>gts_jujutsu_v5_07</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D65" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E65" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F65" t="n">
+        <x:v>10500</x:v>
+      </x:c>
+      <x:c r="G65" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>인물 B 마지막 빈손 포즈 셋업</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>SETUP</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>인물 B가 마지막 공개를 위한 빈손 포즈를 취하고 배경·카메라를 고정</x:v>
+      </x:c>
+      <x:c r="K65" t="str">
+        <x:v>POSE_HOLD_END_ANCHORED; S08과 정렬하고 12000ms SFX 직전에 종료</x:v>
+      </x:c>
       <x:c r="L65"/>
-      <x:c r="M65"/>
-      <x:c r="N65"/>
-      <x:c r="O65"/>
-      <x:c r="P65"/>
-      <x:c r="Q65"/>
-      <x:c r="R65"/>
-      <x:c r="S65"/>
-      <x:c r="T65"/>
-      <x:c r="U65"/>
-      <x:c r="V65"/>
-      <x:c r="W65"/>
+      <x:c r="M65" t="str">
+        <x:v>promo.quaternary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N65" t="str">
+        <x:v>네 번째 실제 메뉴를 놓을 위치를 비워 두고 S08과 동일 인물·구도 유지</x:v>
+      </x:c>
+      <x:c r="O65" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P65" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q65" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R65" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S65" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T65" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U65" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V65" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W65" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="78" customHeight="1">
-      <x:c r="A66"/>
-      <x:c r="B66"/>
-      <x:c r="C66"/>
-      <x:c r="D66"/>
-      <x:c r="E66"/>
-      <x:c r="F66"/>
-      <x:c r="G66"/>
-      <x:c r="H66"/>
-      <x:c r="I66"/>
-      <x:c r="J66"/>
-      <x:c r="K66"/>
+      <x:c r="A66" t="str">
+        <x:v>gts_jujutsu_v5_08</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>gt_jujutsu_transition_v5</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>jujutsu_transition</x:v>
+      </x:c>
+      <x:c r="D66" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E66" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F66" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="G66" t="n">
+        <x:v>14000</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>인물 B 제품 최종 공개</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>MAGIC_REVEAL</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>S07과 동일 포즈·구도에서 실제 제품이 나타난 상태로 전환해 아웃트로 유지</x:v>
+      </x:c>
+      <x:c r="K66" t="str">
+        <x:v>12000ms SFX 타격점 HARD_CUT_MATCH; speed=1.0; 14000ms까지 결과 홀드</x:v>
+      </x:c>
       <x:c r="L66"/>
-      <x:c r="M66"/>
-      <x:c r="N66"/>
-      <x:c r="O66"/>
-      <x:c r="P66"/>
-      <x:c r="Q66"/>
-      <x:c r="R66"/>
-      <x:c r="S66"/>
-      <x:c r="T66"/>
-      <x:c r="U66"/>
-      <x:c r="V66"/>
-      <x:c r="W66"/>
+      <x:c r="M66" t="str">
+        <x:v>promo.quaternary,store.owner_face_allowed</x:v>
+      </x:c>
+      <x:c r="N66" t="str">
+        <x:v>실제 촬영된 제품/상품을 명확히 보여주고 추가 전환 없이 종료</x:v>
+      </x:c>
+      <x:c r="O66" t="str">
+        <x:v>sfx</x:v>
+      </x:c>
+      <x:c r="P66" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q66" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R66" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S66" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T66" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$679:$G$692</x:v>
+      </x:c>
+      <x:c r="U66" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V66" t="str">
+        <x:v>레퍼런스 오디오는 렌더링하지 않고 플랫폼에서 권리 확인된 음원을 추가. 자동 미세 정렬 수치는 서버 정책에서만 해결.</x:v>
+      </x:c>
+      <x:c r="W66" t="str">
+        <x:v>05D8F5E6115DE5C5F237753D3B01AF60EC479E42C2DFA273F2210D6349435FD6</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="78" customHeight="1">
-      <x:c r="A67"/>
-      <x:c r="B67"/>
-      <x:c r="C67"/>
-      <x:c r="D67"/>
-      <x:c r="E67"/>
-      <x:c r="F67"/>
-      <x:c r="G67"/>
-      <x:c r="H67"/>
-      <x:c r="I67"/>
-      <x:c r="J67"/>
-      <x:c r="K67"/>
-      <x:c r="L67"/>
-      <x:c r="M67"/>
-      <x:c r="N67"/>
-      <x:c r="O67"/>
-      <x:c r="P67"/>
-      <x:c r="Q67"/>
-      <x:c r="R67"/>
-      <x:c r="S67"/>
-      <x:c r="T67"/>
-      <x:c r="U67"/>
-      <x:c r="V67"/>
-      <x:c r="W67"/>
+      <x:c r="A67" t="str">
+        <x:v>gts_donggeurio_v1_01</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D67" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E67" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F67" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G67" t="n">
+        <x:v>1033</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>감성 타이틀 훅</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>HOOK</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>안정적인 벽면·공간 디테일을 고정 구도로 보여주고 중앙 프로젝트 타이틀 배치</x:v>
+      </x:c>
+      <x:c r="K67" t="str">
+        <x:v>실측 0~1033ms; 안정 구간 중심 trim; speed 0.95~1.05; 1033ms HARD_CUT</x:v>
+      </x:c>
+      <x:c r="L67" t="str">
+        <x:v>{{project.title}}</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>project.title,store.name</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>레퍼런스 상호·핸들은 복제하지 않고 검증된 프로젝트명/매장명으로 교체</x:v>
+      </x:c>
+      <x:c r="O67" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P67" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q67" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R67" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S67" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T67" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U67" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V67" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W67" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="78" customHeight="1">
-      <x:c r="A68"/>
-      <x:c r="B68"/>
-      <x:c r="C68"/>
-      <x:c r="D68"/>
-      <x:c r="E68"/>
-      <x:c r="F68"/>
-      <x:c r="G68"/>
-      <x:c r="H68"/>
-      <x:c r="I68"/>
-      <x:c r="J68"/>
-      <x:c r="K68"/>
-      <x:c r="L68"/>
-      <x:c r="M68"/>
-      <x:c r="N68"/>
-      <x:c r="O68"/>
-      <x:c r="P68"/>
-      <x:c r="Q68"/>
-      <x:c r="R68"/>
-      <x:c r="S68"/>
-      <x:c r="T68"/>
-      <x:c r="U68"/>
-      <x:c r="V68"/>
-      <x:c r="W68"/>
+      <x:c r="A68" t="str">
+        <x:v>gts_donggeurio_v1_02</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D68" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E68" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F68" t="n">
+        <x:v>1033</x:v>
+      </x:c>
+      <x:c r="G68" t="n">
+        <x:v>3767</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>메뉴 항공샷 공개</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>REVEAL</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>메뉴 전체가 보이는 탑다운/하이앵글 샷에 1.00→1.05 선형 줌인과 하단 보조 텍스트 적용</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>실측 1033~3767ms; 구성 최적 구간 trim; speed 0.9~1.1; 3767ms HARD_CUT</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>{{store.location_or_context}}</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:v>store.location,store.context,promo.primary</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>실제 메뉴와 검증된 장소/맥락만 사용하고 숫자·혜택을 임의 생성하지 않음</x:v>
+      </x:c>
+      <x:c r="O68" t="str">
+        <x:v>caption,text_2d,transform</x:v>
+      </x:c>
+      <x:c r="P68" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q68" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R68" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S68" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T68" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U68" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V68" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W68" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="78" customHeight="1">
-      <x:c r="A69"/>
-      <x:c r="B69"/>
-      <x:c r="C69"/>
-      <x:c r="D69"/>
-      <x:c r="E69"/>
-      <x:c r="F69"/>
-      <x:c r="G69"/>
-      <x:c r="H69"/>
-      <x:c r="I69"/>
-      <x:c r="J69"/>
-      <x:c r="K69"/>
+      <x:c r="A69" t="str">
+        <x:v>gts_donggeurio_v1_03</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D69" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E69" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F69" t="n">
+        <x:v>3767</x:v>
+      </x:c>
+      <x:c r="G69" t="n">
+        <x:v>4700</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>카페 공간 팬</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>AMBIENCE</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>조명·좌석·인테리어를 보여주는 가장 매끄러운 우향 팬/측면 이동 구간 선택</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>실측 3767~4700ms; 모션 중심 trim; speed 0.9~1.35; 소스 팬 보존; 4700ms HARD_CUT</x:v>
+      </x:c>
       <x:c r="L69"/>
-      <x:c r="M69"/>
-      <x:c r="N69"/>
-      <x:c r="O69"/>
-      <x:c r="P69"/>
-      <x:c r="Q69"/>
-      <x:c r="R69"/>
-      <x:c r="S69"/>
-      <x:c r="T69"/>
-      <x:c r="U69"/>
-      <x:c r="V69"/>
-      <x:c r="W69"/>
+      <x:c r="M69" t="str">
+        <x:v>store.interior</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>실제 촬영된 공간 정보량이 높은 구간을 사용하고 긴 팬 전체를 강제 고배속하지 않음</x:v>
+      </x:c>
+      <x:c r="O69" t="str">
+        <x:v>transform</x:v>
+      </x:c>
+      <x:c r="P69" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q69" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R69" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S69" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T69" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U69" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V69" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W69" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="78" customHeight="1">
-      <x:c r="A70"/>
-      <x:c r="B70"/>
-      <x:c r="C70"/>
-      <x:c r="D70"/>
-      <x:c r="E70"/>
-      <x:c r="F70"/>
-      <x:c r="G70"/>
-      <x:c r="H70"/>
-      <x:c r="I70"/>
-      <x:c r="J70"/>
-      <x:c r="K70"/>
+      <x:c r="A70" t="str">
+        <x:v>gts_donggeurio_v1_04</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D70" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E70" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F70" t="n">
+        <x:v>4700</x:v>
+      </x:c>
+      <x:c r="G70" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>메뉴 인터랙션 클로즈업</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>ACTION</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>손이나 도구가 음식에 개입하는 클로즈업에서 동작 시작·피크·종료를 보존</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>실측 4700~7000ms; ACTION_PEAK를 슬롯 58% 부근에 배치; speed 0.9~1.1; 7000ms HARD_CUT</x:v>
+      </x:c>
       <x:c r="L70"/>
-      <x:c r="M70"/>
-      <x:c r="N70"/>
-      <x:c r="O70"/>
-      <x:c r="P70"/>
-      <x:c r="Q70"/>
-      <x:c r="R70"/>
-      <x:c r="S70"/>
-      <x:c r="T70"/>
-      <x:c r="U70"/>
-      <x:c r="V70"/>
-      <x:c r="W70"/>
+      <x:c r="M70" t="str">
+        <x:v>promo.primary.action</x:v>
+      </x:c>
+      <x:c r="N70" t="str">
+        <x:v>실제 촬영된 섞기·집기·서빙 행동을 우선하며 없는 행동을 생성하지 않음</x:v>
+      </x:c>
+      <x:c r="O70" t="str">
+        <x:v>transform</x:v>
+      </x:c>
+      <x:c r="P70" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q70" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R70" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S70" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T70" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U70" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V70" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W70" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="78" customHeight="1">
-      <x:c r="A71"/>
-      <x:c r="B71"/>
-      <x:c r="C71"/>
-      <x:c r="D71"/>
-      <x:c r="E71"/>
-      <x:c r="F71"/>
-      <x:c r="G71"/>
-      <x:c r="H71"/>
-      <x:c r="I71"/>
-      <x:c r="J71"/>
-      <x:c r="K71"/>
+      <x:c r="A71" t="str">
+        <x:v>gts_donggeurio_v1_05</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D71" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E71" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F71" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="G71" t="n">
+        <x:v>8333</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>음식 자르기 액션 하이라이트</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>ACTION_HIGHLIGHT</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>포크/나이프로 음식을 자르거나 분리하는 핵심 순간을 타이트한 클로즈업으로 강조</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>실측 7000~8333ms; ACTION_PEAK 중심 trim; speed 0.75~1.0, 0.8 선호; 8333ms HARD_CUT</x:v>
+      </x:c>
       <x:c r="L71"/>
-      <x:c r="M71"/>
-      <x:c r="N71"/>
-      <x:c r="O71"/>
-      <x:c r="P71"/>
-      <x:c r="Q71"/>
-      <x:c r="R71"/>
-      <x:c r="S71"/>
-      <x:c r="T71"/>
-      <x:c r="U71"/>
-      <x:c r="V71"/>
-      <x:c r="W71"/>
+      <x:c r="M71" t="str">
+        <x:v>promo.secondary.action</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>자르기 장면이 없으면 다른 실제 메뉴 액션으로 대체하고 0.9배 수준까지 완화</x:v>
+      </x:c>
+      <x:c r="O71" t="str">
+        <x:v>transform</x:v>
+      </x:c>
+      <x:c r="P71" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q71" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R71" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S71" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T71" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U71" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V71" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W71" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="78" customHeight="1">
-      <x:c r="A72"/>
-      <x:c r="B72"/>
-      <x:c r="C72"/>
-      <x:c r="D72"/>
-      <x:c r="E72"/>
-      <x:c r="F72"/>
-      <x:c r="G72"/>
-      <x:c r="H72"/>
-      <x:c r="I72"/>
-      <x:c r="J72"/>
-      <x:c r="K72"/>
+      <x:c r="A72" t="str">
+        <x:v>gts_donggeurio_v1_06</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D72" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E72" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F72" t="n">
+        <x:v>8333</x:v>
+      </x:c>
+      <x:c r="G72" t="n">
+        <x:v>9633</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>매장 외관·위치 공개</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>LOCATION</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>매장 외관·간판·입구 등 장소를 식별할 수 있는 구도를 짧게 제시하고 지원될 때만 미세 줌</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>실측 8333~9633ms; 구성 중심 trim; speed 0.9~1.1; 실제 경계는 HARD_CUT 우선</x:v>
+      </x:c>
       <x:c r="L72"/>
-      <x:c r="M72"/>
-      <x:c r="N72"/>
-      <x:c r="O72"/>
-      <x:c r="P72"/>
-      <x:c r="Q72"/>
-      <x:c r="R72"/>
-      <x:c r="S72"/>
-      <x:c r="T72"/>
-      <x:c r="U72"/>
-      <x:c r="V72"/>
-      <x:c r="W72"/>
+      <x:c r="M72" t="str">
+        <x:v>store.name,store.location</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>검증된 매장 외관/위치만 사용하고 SLIDE_LEFT 느낌은 선택적 악센트로만 취급</x:v>
+      </x:c>
+      <x:c r="O72" t="str">
+        <x:v>caption,text_2d,transform</x:v>
+      </x:c>
+      <x:c r="P72" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q72" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R72" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S72" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T72" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U72" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V72" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W72" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="78" customHeight="1">
-      <x:c r="A73"/>
-      <x:c r="B73"/>
-      <x:c r="C73"/>
-      <x:c r="D73"/>
-      <x:c r="E73"/>
-      <x:c r="F73"/>
-      <x:c r="G73"/>
-      <x:c r="H73"/>
-      <x:c r="I73"/>
-      <x:c r="J73"/>
-      <x:c r="K73"/>
+      <x:c r="A73" t="str">
+        <x:v>gts_donggeurio_v1_07</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>gt_donggeurio_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>donggeurio_challenge</x:v>
+      </x:c>
+      <x:c r="D73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F73" t="n">
+        <x:v>9633</x:v>
+      </x:c>
+      <x:c r="G73" t="n">
+        <x:v>12067</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>최종 메뉴 액션 아웃트로</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>OUTRO</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>비비기·들어올리기·떠먹기 등 최종 음식 클로즈업에 1.05→1.00 ease-out 줌아웃</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>실측 9633~12067ms; ACTION_PEAK를 슬롯 48% 부근에 배치; speed 0.9~1.1; 정책값 해소 시에만 FADE_OUT</x:v>
+      </x:c>
       <x:c r="L73"/>
-      <x:c r="M73"/>
-      <x:c r="N73"/>
-      <x:c r="O73"/>
-      <x:c r="P73"/>
-      <x:c r="Q73"/>
-      <x:c r="R73"/>
-      <x:c r="S73"/>
-      <x:c r="T73"/>
-      <x:c r="U73"/>
-      <x:c r="V73"/>
-      <x:c r="W73"/>
+      <x:c r="M73" t="str">
+        <x:v>promo.primary,promo.secondary</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>가장 강한 실제 메뉴 액션을 사용하고 레퍼런스 브랜딩은 복제하지 않음</x:v>
+      </x:c>
+      <x:c r="O73" t="str">
+        <x:v>transform</x:v>
+      </x:c>
+      <x:c r="P73" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q73" t="n">
+        <x:v>46264.395833333336</x:v>
+      </x:c>
+      <x:c r="R73" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S73" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T73" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$693:$G$706</x:v>
+      </x:c>
+      <x:c r="U73" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V73" t="str">
+        <x:v>웜톤 수치·미세 줌·페이드 길이가 미해결이면 서버 정책값 또는 안전한 HARD_CUT/무변형으로 대체. 레퍼런스 브랜드 복제 금지.</x:v>
+      </x:c>
+      <x:c r="W73" t="str">
+        <x:v>197EEB645CBCD97776AAD5D4337EA20074A6DE50BFB0ADDB6F704281A3ABFA5F</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="78" customHeight="1">
       <x:c r="A74"/>

</xml_diff>

<commit_message>
data: add Doma BAD challenge at rank four
</commit_message>
<xml_diff>
--- a/app/template_knowledge/sources/영상편집DB.xlsx
+++ b/app/template_knowledge/sources/영상편집DB.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R2559efaf5987480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R723ce5923351474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="Rb7fe763e7bd64973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R9e0a4e0e15734cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R5efd6aef886f4420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R0fcb1d9fe35340d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="R2300e1cb26c44df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R657d1f5689cb45d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R362a401d4c654592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="Ree13d59270e84394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="Rbd47d9c6a19349cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="Rf769d156e8204fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R4f30a5f5a4c54b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="Raa4fd192d5334f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R527c86b1bd544b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R9d863865b0be4850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="Rc6b30e71dd53416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R1878408dda974f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R0ce19aa02a734138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="Rc28f1779c7f14337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R373a921e9b6b40fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R548f61758e124d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="R75ec71b85e8e4f66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R8420d084a59141f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R896cb77a1b7d415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R4018a0ae05124f9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -959,7 +959,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 세 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
+        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 네 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -1253,16 +1253,16 @@
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>실제 가이드 3종</x:v>
+        <x:v>실제 가이드 4종</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>주술회전 트랜지션 · 동그리오 챌린지 · 오츠카레 썸머 챌린지를 실제 레코드로 등록</x:v>
+        <x:v>주술회전 트랜지션 · 동그리오 챌린지 · 오츠카레 썸머 챌린지 · 도마 BAD 챌린지를 실제 레코드로 등록</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
         <x:v>02, 03, 12</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>12_SOURCE_GUIDES에 세 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
+        <x:v>12_SOURCE_GUIDES에 네 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27276,134 +27276,354 @@
       </x:c>
     </x:row>
     <x:row r="707" ht="18" customHeight="1">
-      <x:c r="A707"/>
-      <x:c r="B707"/>
-      <x:c r="C707"/>
-      <x:c r="D707"/>
-      <x:c r="E707"/>
-      <x:c r="F707"/>
-      <x:c r="G707"/>
-      <x:c r="H707"/>
-      <x:c r="I707"/>
-      <x:c r="J707"/>
-      <x:c r="K707"/>
+      <x:c r="A707" t="str">
+        <x:v>domabad20260831_line_0001</x:v>
+      </x:c>
+      <x:c r="B707" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C707" t="n">
+        <x:v>923</x:v>
+      </x:c>
+      <x:c r="D707" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E707" t="str">
+        <x:v>SUMMARY</x:v>
+      </x:c>
+      <x:c r="F707" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G707" t="str">
+        <x:v>- source_url: https://www.youtube.com/shorts/rUIEHnyoPrU; 11초 STATIC_FULL_SHOT 원테이크, physical_cut_count=0, confidence=0.98, shooting_difficulty: ★★.</x:v>
+      </x:c>
+      <x:c r="H707" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I707" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J707" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K707" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="708" ht="18" customHeight="1">
-      <x:c r="A708"/>
-      <x:c r="B708"/>
-      <x:c r="C708"/>
-      <x:c r="D708"/>
-      <x:c r="E708"/>
-      <x:c r="F708"/>
-      <x:c r="G708"/>
-      <x:c r="H708"/>
-      <x:c r="I708"/>
-      <x:c r="J708"/>
-      <x:c r="K708"/>
+      <x:c r="A708" t="str">
+        <x:v>domabad20260831_line_0002</x:v>
+      </x:c>
+      <x:c r="B708" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C708" t="n">
+        <x:v>924</x:v>
+      </x:c>
+      <x:c r="D708" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E708" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F708" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G708" t="str">
+        <x:v>- 0~4000ms HOOK_SETUP: 고정 전신 구도에서 자연스러운 준비 동작을 연속 수행.</x:v>
+      </x:c>
+      <x:c r="H708" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I708" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J708" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K708" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="709" ht="18" customHeight="1">
-      <x:c r="A709"/>
-      <x:c r="B709"/>
-      <x:c r="C709"/>
-      <x:c r="D709"/>
-      <x:c r="E709"/>
-      <x:c r="F709"/>
-      <x:c r="G709"/>
-      <x:c r="H709"/>
-      <x:c r="I709"/>
-      <x:c r="J709"/>
-      <x:c r="K709"/>
+      <x:c r="A709" t="str">
+        <x:v>domabad20260831_line_0003</x:v>
+      </x:c>
+      <x:c r="B709" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C709" t="n">
+        <x:v>925</x:v>
+      </x:c>
+      <x:c r="D709" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E709" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F709" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G709" t="str">
+        <x:v>- 4000~5000ms PRE_DROP_BUILDUP: 드롭 직전 짧은 준비·방향 전환 동작. 경계에서 영상을 분할하지 않음.</x:v>
+      </x:c>
+      <x:c r="H709" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I709" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J709" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K709" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="710" ht="18" customHeight="1">
-      <x:c r="A710"/>
-      <x:c r="B710"/>
-      <x:c r="C710"/>
-      <x:c r="D710"/>
-      <x:c r="E710"/>
-      <x:c r="F710"/>
-      <x:c r="G710"/>
-      <x:c r="H710"/>
-      <x:c r="I710"/>
-      <x:c r="J710"/>
-      <x:c r="K710"/>
+      <x:c r="A710" t="str">
+        <x:v>domabad20260831_line_0004</x:v>
+      </x:c>
+      <x:c r="B710" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C710" t="n">
+        <x:v>926</x:v>
+      </x:c>
+      <x:c r="D710" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E710" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F710" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G710" t="str">
+        <x:v>- 5000~11000ms CLIMAX_DANCE: 비트 드롭과 동시에 방향을 반전하고 대비되는 안무를 연속 수행.</x:v>
+      </x:c>
+      <x:c r="H710" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I710" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J710" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K710" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="711" ht="18" customHeight="1">
-      <x:c r="A711"/>
-      <x:c r="B711"/>
-      <x:c r="C711"/>
-      <x:c r="D711"/>
-      <x:c r="E711"/>
-      <x:c r="F711"/>
-      <x:c r="G711"/>
-      <x:c r="H711"/>
-      <x:c r="I711"/>
-      <x:c r="J711"/>
-      <x:c r="K711"/>
+      <x:c r="A711" t="str">
+        <x:v>domabad20260831_line_0005</x:v>
+      </x:c>
+      <x:c r="B711" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C711" t="n">
+        <x:v>927</x:v>
+      </x:c>
+      <x:c r="D711" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E711" t="str">
+        <x:v>CONTINUITY</x:v>
+      </x:c>
+      <x:c r="F711" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G711" t="str">
+        <x:v>- ONE_TAKE, expected_take_count_per_output=1, split/reorder/internal trim/start trim/end trim 모두 금지.</x:v>
+      </x:c>
+      <x:c r="H711" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I711" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J711" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K711" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="712" ht="18" customHeight="1">
-      <x:c r="A712"/>
-      <x:c r="B712"/>
-      <x:c r="C712"/>
-      <x:c r="D712"/>
-      <x:c r="E712"/>
-      <x:c r="F712"/>
-      <x:c r="G712"/>
-      <x:c r="H712"/>
-      <x:c r="I712"/>
-      <x:c r="J712"/>
-      <x:c r="K712"/>
+      <x:c r="A712" t="str">
+        <x:v>domabad20260831_line_0006</x:v>
+      </x:c>
+      <x:c r="B712" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C712" t="n">
+        <x:v>928</x:v>
+      </x:c>
+      <x:c r="D712" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E712" t="str">
+        <x:v>CAMERA</x:v>
+      </x:c>
+      <x:c r="F712" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G712" t="str">
+        <x:v>- 전체 STATIC_FULL_SHOT. 카메라 이동, 디지털 줌, animated pan/rotation, punch-in 및 transform keyframe 없음.</x:v>
+      </x:c>
+      <x:c r="H712" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I712" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J712" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K712" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="713" ht="18" customHeight="1">
-      <x:c r="A713"/>
-      <x:c r="B713"/>
-      <x:c r="C713"/>
-      <x:c r="D713"/>
-      <x:c r="E713"/>
-      <x:c r="F713"/>
-      <x:c r="G713"/>
-      <x:c r="H713"/>
-      <x:c r="I713"/>
-      <x:c r="J713"/>
-      <x:c r="K713"/>
+      <x:c r="A713" t="str">
+        <x:v>domabad20260831_line_0007</x:v>
+      </x:c>
+      <x:c r="B713" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C713" t="n">
+        <x:v>929</x:v>
+      </x:c>
+      <x:c r="D713" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E713" t="str">
+        <x:v>AUDIO_SYNC</x:v>
+      </x:c>
+      <x:c r="F713" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G713" t="str">
+        <x:v>- 5000ms VISUAL_DROP_REVERSAL과 AUDIO_DROP_HIT 정렬. 외부 음원이 있을 때 audio offset만 조정하고 영상 타임라인은 유지.</x:v>
+      </x:c>
+      <x:c r="H713" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I713" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J713" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K713" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="714" ht="18" customHeight="1">
-      <x:c r="A714"/>
-      <x:c r="B714"/>
-      <x:c r="C714"/>
-      <x:c r="D714"/>
-      <x:c r="E714"/>
-      <x:c r="F714"/>
-      <x:c r="G714"/>
-      <x:c r="H714"/>
-      <x:c r="I714"/>
-      <x:c r="J714"/>
-      <x:c r="K714"/>
+      <x:c r="A714" t="str">
+        <x:v>domabad20260831_line_0008</x:v>
+      </x:c>
+      <x:c r="B714" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C714" t="n">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="D714" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E714" t="str">
+        <x:v>CAPTION</x:v>
+      </x:c>
+      <x:c r="F714" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G714" t="str">
+        <x:v>- 레퍼런스 자막 근거 없음. 고정 문구를 복제하지 않고 사용자 영상·홍보 맥락에서 동적으로 생성하며 드롭 앵커를 가리지 않음.</x:v>
+      </x:c>
+      <x:c r="H714" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I714" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J714" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K714" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="715" ht="18" customHeight="1">
-      <x:c r="A715"/>
-      <x:c r="B715"/>
-      <x:c r="C715"/>
-      <x:c r="D715"/>
-      <x:c r="E715"/>
-      <x:c r="F715"/>
-      <x:c r="G715"/>
-      <x:c r="H715"/>
-      <x:c r="I715"/>
-      <x:c r="J715"/>
-      <x:c r="K715"/>
+      <x:c r="A715" t="str">
+        <x:v>domabad20260831_line_0009</x:v>
+      </x:c>
+      <x:c r="B715" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C715" t="n">
+        <x:v>931</x:v>
+      </x:c>
+      <x:c r="D715" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E715" t="str">
+        <x:v>INPUT_POLICY</x:v>
+      </x:c>
+      <x:c r="F715" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G715" t="str">
+        <x:v>- 단일 연속 사용자 영상 1개만 사용. 사진, B-roll, cutaway, multi-clip montage는 허용하지 않음.</x:v>
+      </x:c>
+      <x:c r="H715" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I715" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J715" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K715" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="716" ht="18" customHeight="1">
-      <x:c r="A716"/>
-      <x:c r="B716"/>
-      <x:c r="C716"/>
-      <x:c r="D716"/>
-      <x:c r="E716"/>
-      <x:c r="F716"/>
-      <x:c r="G716"/>
-      <x:c r="H716"/>
-      <x:c r="I716"/>
-      <x:c r="J716"/>
-      <x:c r="K716"/>
+      <x:c r="A716" t="str">
+        <x:v>domabad20260831_line_0010</x:v>
+      </x:c>
+      <x:c r="B716" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C716" t="n">
+        <x:v>932</x:v>
+      </x:c>
+      <x:c r="D716" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E716" t="str">
+        <x:v>VALIDATION</x:v>
+      </x:c>
+      <x:c r="F716" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G716" t="str">
+        <x:v>- video span=1, split=false, physical transition=0, speed=1.0, reverse=false, freeze=false, image/B-roll=0, reference caption reuse=false.</x:v>
+      </x:c>
+      <x:c r="H716" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I716" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J716" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K716" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="717" ht="18" customHeight="1">
       <x:c r="A717"/>
@@ -33245,7 +33465,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 세 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 1·2·3위를 유지하며 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>승인된 네 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 1·2·3·4위를 유지하며 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -33276,10 +33496,10 @@
         <x:v>챌린지 입력</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>주술회전 1위·동그리오 2위·오츠카레 썸머 3위</x:v>
+        <x:v>주술회전 1위·동그리오 2위·오츠카레 썸머 3위·도마 BAD 4위</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>02_INPUT_GUIDES</x:v>
@@ -33290,7 +33510,7 @@
         <x:v>전체 가이드 템플릿 구간</x:v>
       </x:c>
       <x:c r="B6" s="5" t="n">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
         <x:v>버전 이력을 포함한 03_GUIDE_TEMPLATES 데이터 행</x:v>
@@ -33388,10 +33608,10 @@
         <x:v>프레임 분석 실행 구간</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>167</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>기존 152개 블록 + 주술회전 8컷 + 동그리오 7컷의 신규 JSON 근거</x:v>
+        <x:v>기존 167개 구간 + 도마 BAD 원테이크의 의미 구간 3개</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -33436,6 +33656,20 @@
         <x:v>실측 0~12.067초의 훅·메뉴·공간·액션·외관·아웃트로 7컷</x:v>
       </x:c>
       <x:c r="D16" t="str">
+        <x:v>03_GUIDE_TEMPLATES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>도마 BAD v1 실행 구간</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>0~11초 단일 연속 촬영 안의 SETUP·BUILDUP·CLIMAX 3개 의미 구간</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
       </x:c>
     </x:row>
@@ -33479,7 +33713,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 주술회전·동그리오·오츠카레 썸머 가이드를 유지합니다. rank 1·2·3을 보존하고 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>승인된 주술회전·동그리오·오츠카레 썸머·도마 BAD 가이드를 유지합니다. rank 1·2·3·4를 보존하고 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -33646,16 +33880,39 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8"/>
-      <x:c r="B8"/>
-      <x:c r="C8"/>
-      <x:c r="D8"/>
-      <x:c r="E8"/>
-      <x:c r="F8"/>
-      <x:c r="G8"/>
-      <x:c r="H8"/>
-      <x:c r="I8"/>
-      <x:c r="J8"/>
+      <x:c r="A8" t="str">
+        <x:v>uploaded_analysis_json_20260831</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>도마 BAD 챌린지</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>도마 BAD 챌린지</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>https://www.youtube.com/shorts/rUIEHnyoPrU</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>rUIEHnyoPrU</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>challenge</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>챌린지</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
@@ -33680,9 +33937,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc3c8540323df46bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R89123a148bde41bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rbfb375263a4c4223"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rb313eb92af034c28"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R3686e214b02c4ebe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rf8b4b3552e5d4972"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -33719,7 +33976,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="119" t="str">
-        <x:v>실제 편집 가이드 3종 · 원본 스키마 고정형 v5.4</x:v>
+        <x:v>실제 편집 가이드 4종 · 원본 스키마 고정형 v5.4</x:v>
       </x:c>
       <x:c r="B1" s="31"/>
       <x:c r="C1" s="31"/>
@@ -33746,7 +34003,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="120" t="str">
-        <x:v>최초 템플릿 구조를 유지해 새 시트·새 열을 추가하지 않습니다. 주술회전·동그리오의 업로드 JSON 근거를 action_pattern·timing_rule에 흡수하고, 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>최초 템플릿 구조를 유지해 새 시트·새 열을 추가하지 않습니다. 도마 BAD 업로드 JSON의 원테이크 의미 구간을 action_pattern·timing_rule에 흡수하고, 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -38711,79 +38968,211 @@
       </x:c>
     </x:row>
     <x:row r="74" ht="78" customHeight="1">
-      <x:c r="A74"/>
-      <x:c r="B74"/>
-      <x:c r="C74"/>
-      <x:c r="D74"/>
-      <x:c r="E74"/>
-      <x:c r="F74"/>
-      <x:c r="G74"/>
-      <x:c r="H74"/>
-      <x:c r="I74"/>
-      <x:c r="J74"/>
-      <x:c r="K74"/>
+      <x:c r="A74" t="str">
+        <x:v>gts_doma_bad_v1_01</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F74" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G74" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>정면 준비 동작 훅</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>HOOK_SETUP</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>고정 전신 구도에서 카메라를 바라보며 자연스러운 준비 동작을 이어가고 인물 전체를 프레임 안에 유지</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>0~4000ms 의미 구간; 원본 영상은 분할하지 않음; speed=1.0; 카메라 이동·디지털 줌·전환 없음</x:v>
+      </x:c>
       <x:c r="L74"/>
-      <x:c r="M74"/>
-      <x:c r="N74"/>
-      <x:c r="O74"/>
-      <x:c r="P74"/>
-      <x:c r="Q74"/>
-      <x:c r="R74"/>
-      <x:c r="S74"/>
-      <x:c r="T74"/>
-      <x:c r="U74"/>
-      <x:c r="V74"/>
-      <x:c r="W74"/>
+      <x:c r="M74" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P74" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q74" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R74" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S74" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T74" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U74" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V74" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W74" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="78" customHeight="1">
-      <x:c r="A75"/>
-      <x:c r="B75"/>
-      <x:c r="C75"/>
-      <x:c r="D75"/>
-      <x:c r="E75"/>
-      <x:c r="F75"/>
-      <x:c r="G75"/>
-      <x:c r="H75"/>
-      <x:c r="I75"/>
-      <x:c r="J75"/>
-      <x:c r="K75"/>
+      <x:c r="A75" t="str">
+        <x:v>gts_doma_bad_v1_02</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D75" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E75" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F75" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="G75" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>드롭 직전 준비 동작</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>PRE_DROP_BUILDUP</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>같은 고정 전신 구도와 연속 동작을 유지하며 비트 드롭 직전의 짧은 준비·방향 전환 동작 수행</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>4000~5000ms 의미 구간; 5000ms 행동 반전 앵커를 준비하되 물리 컷을 만들지 않음; speed=1.0</x:v>
+      </x:c>
       <x:c r="L75"/>
-      <x:c r="M75"/>
-      <x:c r="N75"/>
-      <x:c r="O75"/>
-      <x:c r="P75"/>
-      <x:c r="Q75"/>
-      <x:c r="R75"/>
-      <x:c r="S75"/>
-      <x:c r="T75"/>
-      <x:c r="U75"/>
-      <x:c r="V75"/>
-      <x:c r="W75"/>
+      <x:c r="M75" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O75" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P75" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q75" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R75" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S75" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T75" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U75" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V75" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W75" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="78" customHeight="1">
-      <x:c r="A76"/>
-      <x:c r="B76"/>
-      <x:c r="C76"/>
-      <x:c r="D76"/>
-      <x:c r="E76"/>
-      <x:c r="F76"/>
-      <x:c r="G76"/>
-      <x:c r="H76"/>
-      <x:c r="I76"/>
-      <x:c r="J76"/>
-      <x:c r="K76"/>
+      <x:c r="A76" t="str">
+        <x:v>gts_doma_bad_v1_03</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F76" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="G76" t="n">
+        <x:v>11000</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>반전 안무 클라이맥스</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>CLIMAX_DANCE</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>비트 드롭과 동시에 몸 또는 이동 방향을 크게 반전한 뒤 대비되는 안무를 끝까지 연속 수행</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>5000~11000ms 의미 구간; 5000ms 시각 행동 반전과 외부 음원 드롭을 가능할 때 ±1프레임 이내 정렬; 영상 분할 없음</x:v>
+      </x:c>
       <x:c r="L76"/>
-      <x:c r="M76"/>
-      <x:c r="N76"/>
-      <x:c r="O76"/>
-      <x:c r="P76"/>
-      <x:c r="Q76"/>
-      <x:c r="R76"/>
-      <x:c r="S76"/>
-      <x:c r="T76"/>
-      <x:c r="U76"/>
-      <x:c r="V76"/>
-      <x:c r="W76"/>
+      <x:c r="M76" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O76" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P76" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q76" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R76" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S76" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T76" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U76" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V76" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W76" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="78" customHeight="1">
       <x:c r="A77"/>

</xml_diff>

<commit_message>
data: add 도마 BAD 챌린지 at rank 4 (#84)
Add the uploaded one-take Doma BAD guide to the canonical video-editing database, trendcluster, runtime adapters, workbooks, and tests.
</commit_message>
<xml_diff>
--- a/app/template_knowledge/sources/영상편집DB.xlsx
+++ b/app/template_knowledge/sources/영상편집DB.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="R2559efaf5987480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R723ce5923351474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="Rb7fe763e7bd64973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="R9e0a4e0e15734cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R5efd6aef886f4420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R0fcb1d9fe35340d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="R2300e1cb26c44df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R657d1f5689cb45d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R362a401d4c654592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="Ree13d59270e84394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="Rbd47d9c6a19349cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="Rf769d156e8204fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R4f30a5f5a4c54b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_GUIDE" sheetId="1" r:id="Raa4fd192d5334f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_DASHBOARD" sheetId="2" r:id="R527c86b1bd544b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_INPUT_GUIDES" sheetId="3" r:id="R9d863865b0be4850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GUIDE_TEMPLATES" sheetId="4" r:id="Rc6b30e71dd53416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_SHOOT_AND_CUTS" sheetId="5" r:id="R1878408dda974f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_PRODUCED_VIDEOS" sheetId="6" r:id="R0ce19aa02a734138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_EDIT_RECIPES" sheetId="7" r:id="Rc28f1779c7f14337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_OVERLAYS" sheetId="8" r:id="R373a921e9b6b40fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_USER_OUTPUTS" sheetId="9" r:id="R548f61758e124d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PERFORMANCE" sheetId="10" r:id="R75ec71b85e8e4f66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_POST_TEMPLATES" sheetId="11" r:id="R8420d084a59141f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_MODEL_POLICIES" sheetId="12" r:id="R896cb77a1b7d415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_SOURCE_GUIDES" sheetId="13" r:id="R4018a0ae05124f9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -959,7 +959,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 세 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
+        <x:v>최초 제공 템플릿의 시트·열 구조를 유지합니다. 현재 승인된 네 가이드의 정밀 분석은 03_GUIDE_TEMPLATES 기존 A:W 안에서 관리하고, 프레임 분석은 action_pattern·timing_rule에 흡수합니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -1253,16 +1253,16 @@
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>실제 가이드 3종</x:v>
+        <x:v>실제 가이드 4종</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>주술회전 트랜지션 · 동그리오 챌린지 · 오츠카레 썸머 챌린지를 실제 레코드로 등록</x:v>
+        <x:v>주술회전 트랜지션 · 동그리오 챌린지 · 오츠카레 썸머 챌린지 · 도마 BAD 챌린지를 실제 레코드로 등록</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
         <x:v>02, 03, 12</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>12_SOURCE_GUIDES에 세 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
+        <x:v>12_SOURCE_GUIDES에 네 가이드의 원문·분석 근거를 보존하고 실행 규칙에 연결</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27276,134 +27276,354 @@
       </x:c>
     </x:row>
     <x:row r="707" ht="18" customHeight="1">
-      <x:c r="A707"/>
-      <x:c r="B707"/>
-      <x:c r="C707"/>
-      <x:c r="D707"/>
-      <x:c r="E707"/>
-      <x:c r="F707"/>
-      <x:c r="G707"/>
-      <x:c r="H707"/>
-      <x:c r="I707"/>
-      <x:c r="J707"/>
-      <x:c r="K707"/>
+      <x:c r="A707" t="str">
+        <x:v>domabad20260831_line_0001</x:v>
+      </x:c>
+      <x:c r="B707" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C707" t="n">
+        <x:v>923</x:v>
+      </x:c>
+      <x:c r="D707" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E707" t="str">
+        <x:v>SUMMARY</x:v>
+      </x:c>
+      <x:c r="F707" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G707" t="str">
+        <x:v>- source_url: https://www.youtube.com/shorts/rUIEHnyoPrU; 11초 STATIC_FULL_SHOT 원테이크, physical_cut_count=0, confidence=0.98, shooting_difficulty: ★★.</x:v>
+      </x:c>
+      <x:c r="H707" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I707" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J707" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K707" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="708" ht="18" customHeight="1">
-      <x:c r="A708"/>
-      <x:c r="B708"/>
-      <x:c r="C708"/>
-      <x:c r="D708"/>
-      <x:c r="E708"/>
-      <x:c r="F708"/>
-      <x:c r="G708"/>
-      <x:c r="H708"/>
-      <x:c r="I708"/>
-      <x:c r="J708"/>
-      <x:c r="K708"/>
+      <x:c r="A708" t="str">
+        <x:v>domabad20260831_line_0002</x:v>
+      </x:c>
+      <x:c r="B708" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C708" t="n">
+        <x:v>924</x:v>
+      </x:c>
+      <x:c r="D708" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E708" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F708" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G708" t="str">
+        <x:v>- 0~4000ms HOOK_SETUP: 고정 전신 구도에서 자연스러운 준비 동작을 연속 수행.</x:v>
+      </x:c>
+      <x:c r="H708" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I708" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J708" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K708" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="709" ht="18" customHeight="1">
-      <x:c r="A709"/>
-      <x:c r="B709"/>
-      <x:c r="C709"/>
-      <x:c r="D709"/>
-      <x:c r="E709"/>
-      <x:c r="F709"/>
-      <x:c r="G709"/>
-      <x:c r="H709"/>
-      <x:c r="I709"/>
-      <x:c r="J709"/>
-      <x:c r="K709"/>
+      <x:c r="A709" t="str">
+        <x:v>domabad20260831_line_0003</x:v>
+      </x:c>
+      <x:c r="B709" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C709" t="n">
+        <x:v>925</x:v>
+      </x:c>
+      <x:c r="D709" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E709" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F709" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G709" t="str">
+        <x:v>- 4000~5000ms PRE_DROP_BUILDUP: 드롭 직전 짧은 준비·방향 전환 동작. 경계에서 영상을 분할하지 않음.</x:v>
+      </x:c>
+      <x:c r="H709" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I709" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J709" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K709" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="710" ht="18" customHeight="1">
-      <x:c r="A710"/>
-      <x:c r="B710"/>
-      <x:c r="C710"/>
-      <x:c r="D710"/>
-      <x:c r="E710"/>
-      <x:c r="F710"/>
-      <x:c r="G710"/>
-      <x:c r="H710"/>
-      <x:c r="I710"/>
-      <x:c r="J710"/>
-      <x:c r="K710"/>
+      <x:c r="A710" t="str">
+        <x:v>domabad20260831_line_0004</x:v>
+      </x:c>
+      <x:c r="B710" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C710" t="n">
+        <x:v>926</x:v>
+      </x:c>
+      <x:c r="D710" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E710" t="str">
+        <x:v>SEMANTIC_PHASE</x:v>
+      </x:c>
+      <x:c r="F710" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G710" t="str">
+        <x:v>- 5000~11000ms CLIMAX_DANCE: 비트 드롭과 동시에 방향을 반전하고 대비되는 안무를 연속 수행.</x:v>
+      </x:c>
+      <x:c r="H710" t="str">
+        <x:v>도마BAD_1프레임.json</x:v>
+      </x:c>
+      <x:c r="I710" t="str">
+        <x:v>91A65C9532353963E3F00EC831CC46F59464A361F8A598F2CECBCD2E6E168BA1</x:v>
+      </x:c>
+      <x:c r="J710" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K710" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="711" ht="18" customHeight="1">
-      <x:c r="A711"/>
-      <x:c r="B711"/>
-      <x:c r="C711"/>
-      <x:c r="D711"/>
-      <x:c r="E711"/>
-      <x:c r="F711"/>
-      <x:c r="G711"/>
-      <x:c r="H711"/>
-      <x:c r="I711"/>
-      <x:c r="J711"/>
-      <x:c r="K711"/>
+      <x:c r="A711" t="str">
+        <x:v>domabad20260831_line_0005</x:v>
+      </x:c>
+      <x:c r="B711" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C711" t="n">
+        <x:v>927</x:v>
+      </x:c>
+      <x:c r="D711" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E711" t="str">
+        <x:v>CONTINUITY</x:v>
+      </x:c>
+      <x:c r="F711" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G711" t="str">
+        <x:v>- ONE_TAKE, expected_take_count_per_output=1, split/reorder/internal trim/start trim/end trim 모두 금지.</x:v>
+      </x:c>
+      <x:c r="H711" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I711" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J711" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K711" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="712" ht="18" customHeight="1">
-      <x:c r="A712"/>
-      <x:c r="B712"/>
-      <x:c r="C712"/>
-      <x:c r="D712"/>
-      <x:c r="E712"/>
-      <x:c r="F712"/>
-      <x:c r="G712"/>
-      <x:c r="H712"/>
-      <x:c r="I712"/>
-      <x:c r="J712"/>
-      <x:c r="K712"/>
+      <x:c r="A712" t="str">
+        <x:v>domabad20260831_line_0006</x:v>
+      </x:c>
+      <x:c r="B712" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C712" t="n">
+        <x:v>928</x:v>
+      </x:c>
+      <x:c r="D712" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E712" t="str">
+        <x:v>CAMERA</x:v>
+      </x:c>
+      <x:c r="F712" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G712" t="str">
+        <x:v>- 전체 STATIC_FULL_SHOT. 카메라 이동, 디지털 줌, animated pan/rotation, punch-in 및 transform keyframe 없음.</x:v>
+      </x:c>
+      <x:c r="H712" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I712" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J712" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K712" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="713" ht="18" customHeight="1">
-      <x:c r="A713"/>
-      <x:c r="B713"/>
-      <x:c r="C713"/>
-      <x:c r="D713"/>
-      <x:c r="E713"/>
-      <x:c r="F713"/>
-      <x:c r="G713"/>
-      <x:c r="H713"/>
-      <x:c r="I713"/>
-      <x:c r="J713"/>
-      <x:c r="K713"/>
+      <x:c r="A713" t="str">
+        <x:v>domabad20260831_line_0007</x:v>
+      </x:c>
+      <x:c r="B713" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C713" t="n">
+        <x:v>929</x:v>
+      </x:c>
+      <x:c r="D713" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E713" t="str">
+        <x:v>AUDIO_SYNC</x:v>
+      </x:c>
+      <x:c r="F713" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G713" t="str">
+        <x:v>- 5000ms VISUAL_DROP_REVERSAL과 AUDIO_DROP_HIT 정렬. 외부 음원이 있을 때 audio offset만 조정하고 영상 타임라인은 유지.</x:v>
+      </x:c>
+      <x:c r="H713" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I713" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J713" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K713" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="714" ht="18" customHeight="1">
-      <x:c r="A714"/>
-      <x:c r="B714"/>
-      <x:c r="C714"/>
-      <x:c r="D714"/>
-      <x:c r="E714"/>
-      <x:c r="F714"/>
-      <x:c r="G714"/>
-      <x:c r="H714"/>
-      <x:c r="I714"/>
-      <x:c r="J714"/>
-      <x:c r="K714"/>
+      <x:c r="A714" t="str">
+        <x:v>domabad20260831_line_0008</x:v>
+      </x:c>
+      <x:c r="B714" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C714" t="n">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="D714" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E714" t="str">
+        <x:v>CAPTION</x:v>
+      </x:c>
+      <x:c r="F714" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G714" t="str">
+        <x:v>- 레퍼런스 자막 근거 없음. 고정 문구를 복제하지 않고 사용자 영상·홍보 맥락에서 동적으로 생성하며 드롭 앵커를 가리지 않음.</x:v>
+      </x:c>
+      <x:c r="H714" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I714" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J714" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K714" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="715" ht="18" customHeight="1">
-      <x:c r="A715"/>
-      <x:c r="B715"/>
-      <x:c r="C715"/>
-      <x:c r="D715"/>
-      <x:c r="E715"/>
-      <x:c r="F715"/>
-      <x:c r="G715"/>
-      <x:c r="H715"/>
-      <x:c r="I715"/>
-      <x:c r="J715"/>
-      <x:c r="K715"/>
+      <x:c r="A715" t="str">
+        <x:v>domabad20260831_line_0009</x:v>
+      </x:c>
+      <x:c r="B715" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C715" t="n">
+        <x:v>931</x:v>
+      </x:c>
+      <x:c r="D715" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E715" t="str">
+        <x:v>INPUT_POLICY</x:v>
+      </x:c>
+      <x:c r="F715" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G715" t="str">
+        <x:v>- 단일 연속 사용자 영상 1개만 사용. 사진, B-roll, cutaway, multi-clip montage는 허용하지 않음.</x:v>
+      </x:c>
+      <x:c r="H715" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I715" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J715" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K715" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="716" ht="18" customHeight="1">
-      <x:c r="A716"/>
-      <x:c r="B716"/>
-      <x:c r="C716"/>
-      <x:c r="D716"/>
-      <x:c r="E716"/>
-      <x:c r="F716"/>
-      <x:c r="G716"/>
-      <x:c r="H716"/>
-      <x:c r="I716"/>
-      <x:c r="J716"/>
-      <x:c r="K716"/>
+      <x:c r="A716" t="str">
+        <x:v>domabad20260831_line_0010</x:v>
+      </x:c>
+      <x:c r="B716" t="str">
+        <x:v>uploaded_doma_bad_json_20260831</x:v>
+      </x:c>
+      <x:c r="C716" t="n">
+        <x:v>932</x:v>
+      </x:c>
+      <x:c r="D716" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="E716" t="str">
+        <x:v>VALIDATION</x:v>
+      </x:c>
+      <x:c r="F716" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G716" t="str">
+        <x:v>- video span=1, split=false, physical transition=0, speed=1.0, reverse=false, freeze=false, image/B-roll=0, reference caption reuse=false.</x:v>
+      </x:c>
+      <x:c r="H716" t="str">
+        <x:v>도마BAD_인사이트.json</x:v>
+      </x:c>
+      <x:c r="I716" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
+      <x:c r="J716" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="K716" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS</x:v>
+      </x:c>
     </x:row>
     <x:row r="717" ht="18" customHeight="1">
       <x:c r="A717"/>
@@ -33245,7 +33465,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 세 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 1·2·3위를 유지하며 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>승인된 네 가이드의 실행 구간과 이후 사용자 영상 레코드를 집계합니다. 랭킹 1·2·3·4위를 유지하며 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -33276,10 +33496,10 @@
         <x:v>챌린지 입력</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>주술회전 1위·동그리오 2위·오츠카레 썸머 3위</x:v>
+        <x:v>주술회전 1위·동그리오 2위·오츠카레 썸머 3위·도마 BAD 4위</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
         <x:v>02_INPUT_GUIDES</x:v>
@@ -33290,7 +33510,7 @@
         <x:v>전체 가이드 템플릿 구간</x:v>
       </x:c>
       <x:c r="B6" s="5" t="n">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
         <x:v>버전 이력을 포함한 03_GUIDE_TEMPLATES 데이터 행</x:v>
@@ -33388,10 +33608,10 @@
         <x:v>프레임 분석 실행 구간</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:v>167</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>기존 152개 블록 + 주술회전 8컷 + 동그리오 7컷의 신규 JSON 근거</x:v>
+        <x:v>기존 167개 구간 + 도마 BAD 원테이크의 의미 구간 3개</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
@@ -33436,6 +33656,20 @@
         <x:v>실측 0~12.067초의 훅·메뉴·공간·액션·외관·아웃트로 7컷</x:v>
       </x:c>
       <x:c r="D16" t="str">
+        <x:v>03_GUIDE_TEMPLATES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>도마 BAD v1 실행 구간</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>0~11초 단일 연속 촬영 안의 SETUP·BUILDUP·CLIMAX 3개 의미 구간</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
         <x:v>03_GUIDE_TEMPLATES</x:v>
       </x:c>
     </x:row>
@@ -33479,7 +33713,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="116" t="str">
-        <x:v>승인된 주술회전·동그리오·오츠카레 썸머 가이드를 유지합니다. rank 1·2·3을 보존하고 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>승인된 주술회전·동그리오·오츠카레 썸머·도마 BAD 가이드를 유지합니다. rank 1·2·3·4를 보존하고 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -33646,16 +33880,39 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8"/>
-      <x:c r="B8"/>
-      <x:c r="C8"/>
-      <x:c r="D8"/>
-      <x:c r="E8"/>
-      <x:c r="F8"/>
-      <x:c r="G8"/>
-      <x:c r="H8"/>
-      <x:c r="I8"/>
-      <x:c r="J8"/>
+      <x:c r="A8" t="str">
+        <x:v>uploaded_analysis_json_20260831</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>도마 BAD 챌린지</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>도마 BAD 챌린지</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>https://www.youtube.com/shorts/rUIEHnyoPrU</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>rUIEHnyoPrU</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>challenge</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>챌린지</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
@@ -33680,9 +33937,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc3c8540323df46bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R89123a148bde41bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rbfb375263a4c4223"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rb313eb92af034c28"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R3686e214b02c4ebe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="Rf8b4b3552e5d4972"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -33719,7 +33976,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="119" t="str">
-        <x:v>실제 편집 가이드 3종 · 원본 스키마 고정형 v5.4</x:v>
+        <x:v>실제 편집 가이드 4종 · 원본 스키마 고정형 v5.4</x:v>
       </x:c>
       <x:c r="B1" s="31"/>
       <x:c r="C1" s="31"/>
@@ -33746,7 +34003,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="120" t="str">
-        <x:v>최초 템플릿 구조를 유지해 새 시트·새 열을 추가하지 않습니다. 주술회전·동그리오의 업로드 JSON 근거를 action_pattern·timing_rule에 흡수하고, 카페 추천 리뷰는 포함하지 않습니다.</x:v>
+        <x:v>최초 템플릿 구조를 유지해 새 시트·새 열을 추가하지 않습니다. 도마 BAD 업로드 JSON의 원테이크 의미 구간을 action_pattern·timing_rule에 흡수하고, 삭제된 카페 추천 리뷰는 포함하지 않습니다.</x:v>
       </x:c>
       <x:c r="B2" s="31"/>
       <x:c r="C2" s="31"/>
@@ -38711,79 +38968,211 @@
       </x:c>
     </x:row>
     <x:row r="74" ht="78" customHeight="1">
-      <x:c r="A74"/>
-      <x:c r="B74"/>
-      <x:c r="C74"/>
-      <x:c r="D74"/>
-      <x:c r="E74"/>
-      <x:c r="F74"/>
-      <x:c r="G74"/>
-      <x:c r="H74"/>
-      <x:c r="I74"/>
-      <x:c r="J74"/>
-      <x:c r="K74"/>
+      <x:c r="A74" t="str">
+        <x:v>gts_doma_bad_v1_01</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F74" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G74" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>정면 준비 동작 훅</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>HOOK_SETUP</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>고정 전신 구도에서 카메라를 바라보며 자연스러운 준비 동작을 이어가고 인물 전체를 프레임 안에 유지</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>0~4000ms 의미 구간; 원본 영상은 분할하지 않음; speed=1.0; 카메라 이동·디지털 줌·전환 없음</x:v>
+      </x:c>
       <x:c r="L74"/>
-      <x:c r="M74"/>
-      <x:c r="N74"/>
-      <x:c r="O74"/>
-      <x:c r="P74"/>
-      <x:c r="Q74"/>
-      <x:c r="R74"/>
-      <x:c r="S74"/>
-      <x:c r="T74"/>
-      <x:c r="U74"/>
-      <x:c r="V74"/>
-      <x:c r="W74"/>
+      <x:c r="M74" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P74" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q74" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R74" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S74" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T74" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U74" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V74" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W74" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="78" customHeight="1">
-      <x:c r="A75"/>
-      <x:c r="B75"/>
-      <x:c r="C75"/>
-      <x:c r="D75"/>
-      <x:c r="E75"/>
-      <x:c r="F75"/>
-      <x:c r="G75"/>
-      <x:c r="H75"/>
-      <x:c r="I75"/>
-      <x:c r="J75"/>
-      <x:c r="K75"/>
+      <x:c r="A75" t="str">
+        <x:v>gts_doma_bad_v1_02</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D75" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E75" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F75" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="G75" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>드롭 직전 준비 동작</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>PRE_DROP_BUILDUP</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>같은 고정 전신 구도와 연속 동작을 유지하며 비트 드롭 직전의 짧은 준비·방향 전환 동작 수행</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>4000~5000ms 의미 구간; 5000ms 행동 반전 앵커를 준비하되 물리 컷을 만들지 않음; speed=1.0</x:v>
+      </x:c>
       <x:c r="L75"/>
-      <x:c r="M75"/>
-      <x:c r="N75"/>
-      <x:c r="O75"/>
-      <x:c r="P75"/>
-      <x:c r="Q75"/>
-      <x:c r="R75"/>
-      <x:c r="S75"/>
-      <x:c r="T75"/>
-      <x:c r="U75"/>
-      <x:c r="V75"/>
-      <x:c r="W75"/>
+      <x:c r="M75" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O75" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P75" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q75" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R75" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S75" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T75" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U75" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V75" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W75" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="78" customHeight="1">
-      <x:c r="A76"/>
-      <x:c r="B76"/>
-      <x:c r="C76"/>
-      <x:c r="D76"/>
-      <x:c r="E76"/>
-      <x:c r="F76"/>
-      <x:c r="G76"/>
-      <x:c r="H76"/>
-      <x:c r="I76"/>
-      <x:c r="J76"/>
-      <x:c r="K76"/>
+      <x:c r="A76" t="str">
+        <x:v>gts_doma_bad_v1_03</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>gt_doma_bad_challenge_v1</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>doma_bad_challenge</x:v>
+      </x:c>
+      <x:c r="D76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F76" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="G76" t="n">
+        <x:v>11000</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>반전 안무 클라이맥스</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>CLIMAX_DANCE</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>비트 드롭과 동시에 몸 또는 이동 방향을 크게 반전한 뒤 대비되는 안무를 끝까지 연속 수행</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>5000~11000ms 의미 구간; 5000ms 시각 행동 반전과 외부 음원 드롭을 가능할 때 ±1프레임 이내 정렬; 영상 분할 없음</x:v>
+      </x:c>
       <x:c r="L76"/>
-      <x:c r="M76"/>
-      <x:c r="N76"/>
-      <x:c r="O76"/>
-      <x:c r="P76"/>
-      <x:c r="Q76"/>
-      <x:c r="R76"/>
-      <x:c r="S76"/>
-      <x:c r="T76"/>
-      <x:c r="U76"/>
-      <x:c r="V76"/>
-      <x:c r="W76"/>
+      <x:c r="M76" t="str">
+        <x:v>project.title,promo.context,store.context</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>레퍼런스 인원·복장·자막을 복제하지 않고 사용자 영상과 홍보 맥락에 맞춘 동작·텍스트만 사용</x:v>
+      </x:c>
+      <x:c r="O76" t="str">
+        <x:v>caption,text_2d</x:v>
+      </x:c>
+      <x:c r="P76" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q76" t="n">
+        <x:v>46264.99015046296</x:v>
+      </x:c>
+      <x:c r="R76" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="S76" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="T76" t="str">
+        <x:v>'12_SOURCE_GUIDES'!$G$707:$G$716</x:v>
+      </x:c>
+      <x:c r="U76" t="str">
+        <x:v>UPLOADED_JSON_ANALYSIS_IN_12_SOURCE_GUIDES</x:v>
+      </x:c>
+      <x:c r="V76" t="str">
+        <x:v>단일 연속 영상은 분할·재배열·속도 변경·역재생·프리즈·합성 전환·애니메이션 변형을 금지. 외부 챌린지 음원이 없으면 오디오 재정렬을 생략하고 플랫폼에서 사용자가 권리 확인된 음원을 추가.</x:v>
+      </x:c>
+      <x:c r="W76" t="str">
+        <x:v>B8C30708E56C22517FF97A1ECB76C173EE3A97D91E01175DF37759BFFAA8F78D</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="78" customHeight="1">
       <x:c r="A77"/>

</xml_diff>